<commit_message>
Nachtlauf: 36 Handwerksbetriebe aus Würzburg ergänzen.
Die Suche bleibt auf Maler, Elektriker, Gebäudereinigung und verwandtes Bauhandwerk begrenzt. Bereits gespeicherte Firmen bleiben in der Tabelle.

Co-authored-by: teamtrack1019 <teamtrack1019@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$P$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$P$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P41"/>
+  <dimension ref="A1:P77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3634,8 +3634,2668 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Röder Schlosserei und Montagebau</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>info@roeder-metallbau.de</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>joachim.roeder@t-online.de</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>0931 / 93263</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://www.roeder-metallbau.de</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>https://www.roeder-metallbau.de/kontakt/anfahrt</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>49.830903</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>9.908089</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>node/345622383</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>FERSCH malt</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Maler / Lackierer</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>ferschmalt@ferschmalt.de</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>+49 9302 1223</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Hinterer Talweg 2</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>97228</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Rottendorf</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://www.ferschmalt.de/</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>https://www.ferschmalt.de/</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>49.790154</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>10.021764</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>node/1002783813</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Fensterbau Zinnhobel</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Glaserei</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Karl Jürgen Zinnhobel</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>fensterbau-zinnhobel@t-online.de</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>+49 931 9917360</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Karmelitenstraße 1</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>97070</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://www.zinnhobel.de/</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>https://www.zinnhobel.de/impressum.html</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>49.793303</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>9.927492</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>node/1333961772</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Ziegler Heizungs- und Regelungstechnik GmbH</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>info@ziegler-shk.de</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>info@ieq-systems-shk.de</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>+49931272667</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Friedrich-Bergius-Ring 7</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>97076</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://www.ziegler-shk.de/</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>https://www.ziegler-shk.de/unternehmen/shk/kontakt</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>49.802874</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>9.996240</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>node/2083616143</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Conzept Bad</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Fliesenleger</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Andreas Köstner</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>info@conzept-bad.de</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>0931 - 20 53 53 0</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>https://www.conzept-bad.de</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>https://www.conzept-bad.de/baeder_studio/kontakt/</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>49.795869</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>9.939681</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>node/2477796657</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Hilpert-Heizung Sanitär</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Hilpert Heizung Sanitär Verwaltungs</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>info@hilpert-heizung.de</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>+49 931 79780 0</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Werner-von-Siemens-Straße 16</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>97076</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>https://www.hilpert-heizung.de/</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>https://hilpert-heizung.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>49.798999</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>9.978949</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>node/3806967759</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Elektro-Pixis GmbH</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Tim Pixis</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>info@pixis.de</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>+49 931 70560-0</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Am Kirschberg 4</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>97218</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Gerbrunn</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>https://www.pixis.de/</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>https://www.pixis.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>49.786620</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>9.986598</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>node/4347753904</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Götz Schlüsseldienst</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Schlüsseldienst</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>info@schluessel-goetz.de</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>+49 931 53525</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>97070</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>https://www.schluessel-goetz.de/</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>https://www.schluessel-goetz.de/kontakt</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>49.796827</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>9.928748</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>node/4527142906</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>SIMON Schuhwerkstatt/Schlüsseldienst/Näherei</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Schlüsseldienst</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Gorgette ÜN</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>simonschluesseldienst1983@gmail.com</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>uen83@web.de</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>+49 171 8067034</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Dominikanerpassage 36-38</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>97070</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>https://www.simon-schluesseldienst.de/</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>https://www.simon-schluesseldienst.de/impressum</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>49.796480</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>9.930230</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>node/4784496300</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Elektro Sondheimer</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Manfred Sondheimer</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>info@sondheimer.net</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>mail@universalschlichtungsstelle.de</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>+49 9365 80840</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://sondheimer-elektro.ihr-elektrofachmann.de/</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>https://sondheimer-elektro.ihr-elektrofachmann.de/kontakt/impressum</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>49.846143</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>9.965965</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>node/6610562528</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Martin Weber Haustechnik</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>office@weber-martin.de</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>0931 / 7840947</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>https://www.weber-martin.de</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>https://weber-martin.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>49.795666</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>9.846836</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>node/7448561107</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Thomas Stierhof Wand &amp; Wohnkultur</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Maler / Lackierer</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Thomas Stierhof</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>info@stierhof-wandkultur.com</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>info@stierhof-wandkultur.de</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>+49 931 6193907</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Kurze Gasse 10</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>97076</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>http://www.stierhof-wandkultur.com/</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>http://www.stierhof-wandkultur.com/</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>49.810103</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>9.986360</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>node/8033171794</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Steinwelten Josef Hofmann</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Steinmetz</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Josef Hofmann</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>info@stein-welten.com</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>+49 931 20029 0</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Versbacher Straße 104</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>97078</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>https://stein-welten.com/</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>https://www.stein-welten.com/impressum</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>49.815567</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>9.962790</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>node/8652947771</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Heckelmann &amp; Kirchner</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Zimmerei / Schreinerei</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Christian Heckelmann</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>info@heckelmann-kirchner.de</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>0931 / 27 049 700</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Georg-Engel-Straße 23</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>97076</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://www.heckelmann-kirchner.de</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>https://www.heckelmann-kirchner.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>49.809230</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>9.990250</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>node/8715562395</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Holzbau Preuß &amp; Burkholz</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Zimmerei / Schreinerei</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>+49 931 8807997</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Werner-von-Siemens-Straße 44</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>97076</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>https://hbp.3c7.de/zimmerei-wuerzburg.php</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>https://hbp.3c7.de/zimmerei-wuerzburg.php</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>49.801921</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>9.979598</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>node/8735913718</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>ohne Kontaktdaten</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Porzner</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Dipl.-Ing. Thomas Porzner</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>info@porzner.com</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>+49 931 461234</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Hauptstraße 130</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>https://www.porzner.com</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>https://www.porzner.com/impressum</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>49.809700</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>9.872142</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>node/9035821753</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Moritz Würzburg</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Herrn Armin Hebig</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>info@moritz-wuerzburg.de</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>+49 931 797810</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Randersackerer Straße 51</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>97072</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>https://www.moritz-wuerzburg.de</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>https://moritz-wuerzburg.de/index.php/impressum</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>49.776472</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>9.941535</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>node/9682761730</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Neumüller</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Fensterbau</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>info@fenster-neumueller.de</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>+49 931 30196635</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>https://www.fenster-neumueller.de</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>https://www.fenster-neumueller.de/impressum</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>49.741840</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>9.963851</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>node/9820749556</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>mainTisch</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Schreinerei</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>info@maintisch.de</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>+49 1512 0101070</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>https://maintisch.de</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>https://maintisch.de/kontakt/</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>49.831154</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>9.898286</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>node/9914428513</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Malermeisterbetrieb Walter &amp; Breunig</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Innenausbau</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Markus Walter</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>info@walter-breunig.de</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>+49 931 80996910</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>https://www.walter-breunig.de</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>https://www.walter-breunig.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>49.834717</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>9.907384</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>node/9914429120</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>HESSELBARTH – Gebäude- und Energietechnik</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>info@hesselbarth-get.de</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>+49 931 304296 0</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Daimlerstraße 7</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>97209</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Veitshöchheim</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>https://www.elektro-team.info/</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>https://www.hesselbarth.energy/impressum-2/</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>49.830765</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>9.901219</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>node/9914429196</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Zimmerei Geiger GmbH</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Zimmerei / Schreinerei</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Matthias Geiger</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>info@zimmerei-geiger.de</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>+49 931 45249800</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>https://www.zimmerei-geiger.de</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>https://www.zimmerei-geiger.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>49.831325</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>9.908106</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>node/9914429275</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Flammersberger GmbH Metallbau</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Karl Flammersberger</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>info@flammersberger.com</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>+49 931 970090</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>https://www.flammersberger.de</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>https://flammersberger.de/impressum</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>49.830168</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>9.908210</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>node/9914429277</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Franz Frisch GmbH</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Maler / Lackierer</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Stefan Frisch</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>info@frisch-malerservice.de</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>datenschutz@frisch-malerservice.de</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>0931 / 94698</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>https://www.frisch-malerservice.de</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>https://www.frisch-malerservice.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>49.831796</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>9.904592</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>node/9914429296</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>WPB Würzburger Pflasterbau GmbH</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Pflasterbau</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Ulrich Schätzlein</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>info@wuerzburger-pflasterbau.de</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>+49 931 980690</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>https://www.wuerzburger-pflasterbau.de</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>https://www.wuerzburger-pflasterbau.de/impressum</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>49.832987</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>9.900066</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>node/9914429304</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>alfred rexroth Metallbearbeitung GmbH</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>https://www.rexroth-metallbearbeitung.de/</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>https://www.rexroth-metallbearbeitung.de/</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>49.832642</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>9.899619</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>node/9914429305</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>ohne Kontaktdaten</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Glaserei Nagel</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Glaserei</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Harald Nagel</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>info@glaserei-nagel.de</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>0931 - 26 43 4</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Steinheilstraße 3</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>97080</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>https://www.glaserei-nagel.de/</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>https://www.glaserei-nagel.de/index.php/impressum</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>49.803499</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>9.941102</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>node/10073439309</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Schumann-Kreativwerkstatt</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Zimmerei / Schreinerei</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Anke Lederer</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>info@schumann-kreativwerkstatt.de</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>+49 931 78023 516</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Margetshöchheimer Straße 91</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>97299</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Zell a. Main</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>https://elsol-relax.de/</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>https://schumann-kreativwerkstatt.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>49.821196</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>9.867252</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>node/10159153943</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>fliesenlazar</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Fliesenleger</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>info@fliesenlazar.de</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>+49 931 35820198</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>https://www.fliesenlazar.de/</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>https://www.fliesenlazar.de/kontakt/</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>49.795506</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>9.896818</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>node/10270138356</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Rügamer Gebäudereinigung GmbH</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Gebäudereinigung</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>ruegamer.gebaeudeservice@gmx.net</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>+49 931 53166</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Juliuspromenade 13</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>97070</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>https://www.ruegamer-gebaeudereinigung.de</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>https://www.ruegamer-gebaeudereinigung.de/kontakt</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>49.796950</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>9.929101</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>node/11212253728</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Viessmann</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Thomas Donato</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>info@viessmann-climatesolutions.com</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>+4993161550</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>97076</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>https://www.viessmann.de/de/kontakt/niederlassungen/verkaufsniederlassung-wuerzburg.html</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>https://www.viessmann.de/de/impressum.html</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>49.802137</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>9.997253</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>node/11665645170</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Kimmel GmbH</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>info@kimmel-gmbh.de</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>+49 931 99135900</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Zeller Straße 17</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>97276</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Margetshöchheim</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>https://www.kimmel-gmbh.de/</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>https://www.kimmel-gmbh.de/</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>49.824914</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>9.867881</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>node/11739052818</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Fritz Meder GmbH &amp; Co. KG und FMW-Vertriebs-GmbH</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Fliesenleger</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Heiko Scherbantin</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>info@fmeder.de</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>+49 931 42539</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Daimlerstraße 8</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>97082</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>https://www.fmeder.de/</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>https://www.fmeder.de/www-fmeder-de/impressum</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>49.798996</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>9.906430</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>node/14181078835</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Beck Elektrotechnik GmbH</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Christine Beck-Meidt</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>info@beck-elektrotechnik.de</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>+49 931 20050</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Nürnberger Straße 109</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>97076</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>https://www.team-elektro-beck.de/beck-elektrotechnik-gmbh/leistungen</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>https://www.team-elektro-beck.de/beck-elektrotechnik-gmbh/impressum.html</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>49.799077</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>9.992376</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>way/118635730</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Elektro Ziegler</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Daniel Ziegler</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>info@ziegler-elektroservice.de</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>mail@universalschlichtungsstelle.de</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>+49 93162828</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Klingenstraße 52</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>97084</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>https://www.ziegler-elektroservice.de</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>https://www.ziegler-elektroservice.de/kontakt/impressum</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>49.763057</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>9.945090</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>way/177696029</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Malergeschäft Heckelmann</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Maler / Lackierer</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Bernd Heckelmann</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>info@maler-heckelmann.de</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>inf@maler-heckelmann.de</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>+49 931 271890</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Friedrich-Bergius-Ring 9b</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>97076</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>https://www.maler-heckelmann.de/</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>https://www.maler-heckelmann.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>49.803320</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>9.995667</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>way/202952686</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P41"/>
+  <autoFilter ref="A1:P77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Nachtlauf: 31 Handwerksbetriebe von Würzburg bis Obernburg ergänzen.
Co-authored-by: teamtrack1019 <teamtrack1019@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$P$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$P$108</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P77"/>
+  <dimension ref="A1:P108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -6294,8 +6294,2350 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Steinwerk Haas</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Steinmetz</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>info@steinwerk-haas.de</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>haas@steinwerk-haas.de; hofmann@steinwerk-haas.de; mangold@steinwerk-haas.de</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>+49 931 65347</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Winterhäuser Straße 93</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>97084</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>https://www.steinwerk-haas.de/</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>https://steinwerk-haas.de/kontakt/</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>49.756552</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>9.974696</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>way/231362855</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Wagner Sicherheitstechnik GmbH &amp; Schlüssel Wagner GmbH</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Schlüsseldienst</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Loos Rechtsanwälte</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>info@wagner-sicherheit.de</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>support@wagner-sicherheit.de; datenschutz@wagner-sicherheit.de; info@kanzlei-loos.de</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>+49 931 70588 0</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Käthe-Kollwitz-Straße 3</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>97218</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Gerbrunn</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>https://www.wagner-sicherheit.de/</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>https://www.wagner-sicherheit.de/impressum.html</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Würzburg</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>49.786601</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>9.984000</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>way/321049773</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Schreinerei Walk GmbH</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Zimmerei / Schreinerei</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>der Schreinerei Walk</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>mw@schreinerei-walk.de</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>+49 9306 1376</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Guttenberger Straße 9a</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>97270</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Kist</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>https://www.schreinerei-walk.de/</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>https://www.schreinerei-walk.de/impressum-und-datenschutzerklaerung/</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Kist</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>49.744506</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>9.847993</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>node/7264996813</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>RMS Metalwork GmbH</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Kevin Guhr</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>service@rms-metalwork.de</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>+49 9306 8599</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Sonnleite 15</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>97270</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Kist</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>https://www.rms-metalwork.de/</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>https://rms-metalwork.de/</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Kist</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>49.737562</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>9.842931</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>node/9851405107</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>DGM Deutsche Glas Manufaktur GmbH</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Glaserei</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>info@deutschesglas.de</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>info@funky-bits.de</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>+49 9369 984 96 11</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Prinz-Ludwig-Straße 6</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>97264</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Helmstadt</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>https://www.deutschesglas.de/</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>https://www.deutschesglas.de/#kontakt-datenschutz.html</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Helmstadt</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>49.758719</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>9.716972</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>node/6737950822</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Blank Bauunternehmung</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Bauunternehmen</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Christoph Blank</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>info@bauunternehmung-blank.de</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>+49 9369 1666</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Prinz-Ludwig-Straße 4</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>97264</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Helmstadt</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>https://www.bauunternehmung-blank.de/</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>https://www.bauunternehmung-blank.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Helmstadt</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>49.758934</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>9.716330</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>node/13716960216</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Rumoboden</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Bodenleger</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Christoph Ruhland</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>09342- 935 -</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Carl-Jacob-Kolb-Weg 5</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>97877</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Wertheim</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>https://www.rumoboden.de</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>https://www.rumoboden.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Wertheim</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>49.783864</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>9.506873</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>node/14157163707</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>nur Geschäftsführer</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Heim</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Steinmetz</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Andreas Heim</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>mail@heim-natursteine.de</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>t.giegerich@heim-natursteine.de</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>+49 9371 3112</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Hans-Stiglitz-Weg 2</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>63897</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>https://www.heim-natursteine.de/</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>https://heim-natursteine.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>49.703652</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>9.268454</t>
+        </is>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>node/6777562113</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Felix Bauer Edelstahltechnik</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Felix Bauer</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>info@felix-bauer.com</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>+49 9371 948939 0</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Siemensstraße 5</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>63897</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>https://www.felix-bauer.com</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>https://www.felix-bauer.com/about/</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>49.709329</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>9.244263</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>node/6813758058</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Fliesen-Center Hawel</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Fliesenleger</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Achim Hawel</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>+49 9371 8422</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Oberer Steffleinsgraben 4</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>63927</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Bürgstadt</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>https://www.fliesen-hawel.de/</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>https://www.fliesen-hawel.de/about/</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>49.708703</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>9.267510</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>node/7611578458</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>nur Geschäftsführer</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>F.J.-Riegel</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Stuckateur</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Michael Riegel</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>info@maler-riegel.de</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>+49 9371 1281</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Hauptstraße 58</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>63927</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Bürgstadt</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://www.maler-riegel.de</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>https://www.maler-riegel.de/</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>49.712581</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>9.268718</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>node/8554600522</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>A&amp;R Wachtel</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Maler / Lackierer</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Timo Wachtel</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>timo@malerwachtel.de</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>ralf.wachtel@freenet.de</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>+49 9371 67764</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>http://www.malerwachtel.de</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>http://www.malerwachtel.de/impressum.html</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>49.708837</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>9.268086</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>node/8578245226</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Dietz</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>peter@dietz-metallbau.de</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>+49 171 1719889</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>http://www.dietz-metallbau.de</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>http://www.dietz-metallbau.de/</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>49.725433</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>9.225556</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>node/8594624216</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>FZ Elektrotechnik</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>franz-zoeller@fz-elektro.de</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>+49 9371 682 82</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Ludwigstraße 7</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>63920</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Großheubach</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://www.fz-elektro.de</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>https://www.fz-elektro.de</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>49.728481</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>9.224399</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>node/8618598207</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>CS Clean Service</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Gebäudereinigung</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Sven Klapper</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>info@cs-mil.de</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>+49 9371 657 79</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>https://www.cs-mil.de</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>https://www.cs-mil.de/impressum</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>49.715254</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>9.235090</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>node/8628352047</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>TA Elektrotechnik</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>firma@ta-elektrotechnik.de</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>+49 9371 601 7125</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>https://www.ta-elektrotechnik.de</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>https://www.ta-elektrotechnik.de</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>49.717845</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>9.231268</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>node/8634672157</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Jäger &amp; Kaufmann</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Ronald Jäger</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>info@jaeger-kaufmann.de</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>info@stw-webdesign.de</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>09371 4815</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Im Steiner 20</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>63924</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Kleinheubach</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>https://www.jaeger-kaufmann.de/</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>https://www.jaeger-kaufmann.de/pages/impressum.php</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>49.713463</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>9.223662</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>node/8755631725</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Schneider Innen.Raum.Design</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Schreinerei</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Martin Schneider</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>info@schneider-raum.de</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>09371/94730-0</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Im Bruch 1</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>https://www.schneider-raum.de</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>https://www.schneider-raum.de/impressum.html</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>49.706376</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>9.229564</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>node/9696025927</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>AKS GmbH</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Ahmet Kocyigit</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>info@ak-s.tv</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>anfrage@main-pv.de</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Lassallestraße 7</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>https://ak-s.tv/</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>https://main-pv.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>49.704678</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>9.228066</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>node/10937626870</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Breitenbach Stahl- und Metallbau</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>info@breitenbach-metall.de</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>myjob@breitenbach-metall.de</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>+49 9371 9783-0</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Im Bruch 11</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>63897</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>https://breitenbach-metall.com/</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>https://breitenbach-metall.com/impressum.html</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>49.705074</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>9.227590</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>node/11071021566</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Elektroservice Reichl</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Frank Reichl</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>kontakt@elektroservice-reichl.de</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>mail@universalschlichtungsstelle.de</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>+49 9372 923856</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>https://www.elektroservice-reichl.de</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>https://www.elektroservice-reichl.de/kontakt/impressum</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>49.726381</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>9.221474</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>node/13768610630</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Heim Steintechnik</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Steinmetz</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Martin Heim</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>info@heim-steintechnik.de</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>09371 668010</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Industriestraße 4b</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>63927</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Bürgstadt</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>https://www.heim-steintechnik.de</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>https://www.heim-steintechnik.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>49.731803</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>9.273825</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>way/86264621</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Hefner</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Bodenleger</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Jürgen Hefner</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>info@hefner-boden.de</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>0 93 71 - 94 99 480</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Eichenbühler Straße 89</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>63927</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Bürgstadt</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>https://hefner-boden.de</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>https://hefner-boden.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>Miltenberg</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>49.704187</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>9.281114</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>way/204037343</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Fichtl Holz Hand Werk</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Schreinerei</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>info@schreiner-fichtl.de</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>+49 6022 2086113</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Im Weidig 37</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>63785</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>https://www.schreiner-fichtl.de</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>https://www.schreiner-fichtl.de/kontakt/</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>49.834838</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>9.119144</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>node/3834420811</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>RAKU Stahl &amp; Aluminium GmbH</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Bernd Reichert</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>info@raku-gmbh.de</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>+49 6022 9073</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Spessartstraße 21</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>63785</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>https://www.raku-gmbh.de</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>https://www.raku-gmbh.de/impresum.html</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>49.833422</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>9.118399</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>node/4018673857</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Rehm Trockenbau</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Bauunternehmen</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Michael Rehm</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>info@rehm-trockenbau.de</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>+49 6022 5072011</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Spessartstraße 21</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>63785</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>https://rehm-trockenbau.de/</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>https://rehm-trockenbau.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>49.833397</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>9.118401</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>node/4018673858</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Bausysteme Wagner</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Fensterbau</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>pwagner@wagner-bausysteme.com</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>+49 6022 5067444</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Obernburger Straße 36</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>63853</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Mömlingen</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>https://www.wagner-bausysteme.de</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>https://www.wagner-bausysteme.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>49.851060</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>9.088498</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>node/5624671527</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>ms: Elektrotechnik</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Michael Stegmann</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>info@ms-elektro-technik.de</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>+49 6022 710100</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Im Höning 20</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>https://www.ms-elektro-technik.de</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>https://www.ms-elektro-technik.de/impressum.html</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>49.855620</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>9.167251</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>node/6270137880</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Elektrotechnik Wahl</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr"/>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>+49 9372 940239</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Pfützenäcker 14</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>63906</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Erlenbach am Main</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>https://www.etechnik-wahl.de</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>https://www.etechnik-wahl.de/</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>49.807048</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>9.159334</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>node/7955913151</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>ohne Kontaktdaten</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Heizung Sanitär Kelpetin</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Fatih Kelpetin</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>info@kelpetin.eu</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>+4915141912358</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Liebigstraße 10</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>63906</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Erlenbach am Main</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>https://www.kelpetin.eu/</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>https://www.kelpetin.eu/impressum</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>49.808102</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>9.150558</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>node/9183896147</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Fath Bau</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Bauunternehmen</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Robin Fath</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>info@fath-bau.com</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>+49 170 9129431</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>https://www.fath-bau.com/</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>https://www.fath-bau.com/Impressum</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>49.833786</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>9.120337</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>node/11242169782</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P77"/>
+  <autoFilter ref="A1:P108"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Nachtlauf: 25 Handwerksbetriebe von Kleinheubach bis Aschaffenburg ergänzen.
Co-authored-by: teamtrack1019 <teamtrack1019@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$P$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$P$133</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P108"/>
+  <dimension ref="A1:P133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -8636,8 +8636,1858 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Zwissler</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Heinrich Zwissler</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>buero@zwissler.eu</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>+49 9371 3909</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Rathausstraße</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>63920</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Großheubach</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>https://www.zwissler.eu</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>https://zwissler.eu/index.php/impressum/</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>Kleinheubach</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>49.726475</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>9.220942</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>node/1035407239</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>TW Elektrotechnik – Thomas Waigand</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr"/>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>kontakt@tw-elektrotechnik.com</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>+49 6022 6524389</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Im Höning 12</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>63820</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Elsenfeld</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>https://www.tw-elektrotechnik.com</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>https://www.tw-elektrotechnik.com/</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>49.854641</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>9.166076</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>node/12043664366</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Färber</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Hans-Peter Färber</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>info@faerbergmbh.de</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>06022/71094-0 -</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Grundtalring 16</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>63868</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Großwallstadt</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>https://www.faerbergmbh.de</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>https://www.faerbergmbh.de/anbieterkennzeichnung</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>49.875748</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>9.148984</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>way/280507427</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Zimmerei Boneberger</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Zimmerei / Schreinerei</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr"/>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>info@zimmerei-boneberger.de</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>+49 6022 2233</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>An der Wehrinsel 1</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>63785</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>https://zimmerei-boneberger.de</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>https://zimmerei-boneberger.de/kontakt.html</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>49.831847</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>9.129020</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>way/612232377</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Malerforum HMD GmbH</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Maler / Lackierer</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Patrick Hein</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>info@malerforum.com</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>+49 6022 7093330</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Im Höning 5-9</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>63820</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Elsenfeld</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>https://www.malerforum.com</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>https://www.malerforum.com/impressum/</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>49.854809</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>9.165384</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>way/669564361</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Schreinerei Appel</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Schreinerei</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Julia Brenner</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>+49 6022 2631-0</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Toni-Schecher-Straße 2-4</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>63820</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Elsenfeld</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>https://www.appel-rueck.de</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>https://www.appel-rueck.de/impressum.html</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>49.836481</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>9.193750</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>way/768315260</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>nur Geschäftsführer</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Löwe</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Fensterbau</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Leo Löffler</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>info@loewe-fenster.de</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>+49 6022 6630-0</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>https://www.loewe-fenster.de</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>https://loewe-fenster.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>49.857181</t>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>9.183449</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>way/814968079</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Roth Elektrotechnik</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr"/>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>info@roth-elektrotechnik.com</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>+49 6022 2655880</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Grundtalring 45</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>https://www.roth-elektrotechnik.com</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>https://roth-elektrotechnik.com/kontakt</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>49.876076</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>9.148238</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>way/926308994</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Schreinerei ML</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Schreinerei</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr"/>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>info@schreinereiml.com</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>info@schreinereiml.de</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>+49 9372 9444383</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Dr.-Gammert-Straße 21</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>63906</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Erlenbach am Main</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>https://www.schreinereiml.com/</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>https://www.schreinereiml.com/kontakt</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>49.819423</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>9.154656</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>way/1036095393</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Schreinerei Hammerbacher</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Zimmerei / Schreinerei</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Stephan Hammerbacher</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>info@schreinerei-hammerbacher.de</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>+49 (0) 6021 / 2 25 96</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>https://www.schreinerei-hammerbacher.de/</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>https://www.schreinerei-hammerbacher.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>49.966022</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>9.142354</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>node/3502669717</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Steinwerk Hirte</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Steinmetz</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr"/>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>info@steinwerk-hirte.de</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>06021 929485</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>https://www.stein-werk.eu/</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>https://www.steinwerk-hirte.de/impressum</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>49.970633</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>9.147959</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>node/3535241018</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Ludwig Meister</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Elisabeth Meister</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>info@ludwigmeister.de</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>dachau@ludwigmeister.de; aschaffenburg@ludwigmeister.de; augsburg@ludwigmeister.de</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>+49 8131 / 3331 - 0</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Magnolienweg 31</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>63741</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>https://www.ludwigmeister.de/unternehmen/standorte</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>https://www.ludwigmeister.de/impressum</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>49.968550</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>9.131222</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>node/3719664430</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Ulltech AG</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Michael Roth</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>info@ulltech-ag.de</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>06021-386530</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>https://www.ulltech.de/</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>https://ulltech.de/impressum</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>49.968312</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>9.132410</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>node/3719664440</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Glasstudio Bergmann</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Glaserei</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Susanne Dreisbusch</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>info@glasstudio-bergmann.de</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>+49 6021 28484</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>https://www.glasstudio-bergmann.de/</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>https://glasstudio-bergmann.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>49.977447</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>9.142295</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>node/3822522222</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Benedict Systemtechnik GmbH</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Gottfried Köhler</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>info@benedict-gmbh.de</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>+49 (0)6021</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>https://www.benedict-gmbh.de/</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>https://www.benedict-gmbh.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>49.987561</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>9.107518</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>node/3945499136</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Günther Kälte-Klima GmbH</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Peter Hoffmann</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>kontakt@gkk.net</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>+49-6021-34940</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>https://www.gkk.net/</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>https://www.gkk.net/ueber-uns/</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>49.985115</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>9.121865</t>
+        </is>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>node/4151156078</t>
+        </is>
+      </c>
+      <c r="P124" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Elektro Max</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr"/>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>mail@universalschlichtungsstelle.de</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>elektromax@online.de</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>06021/5851666</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>https://www.elektromax-hausgeraete.de/</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>https://www.elektromax-hausgeraete.de/kontakt/kontaktformular</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>49.990569</t>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>9.134935</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>node/4328998175</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Adam Höflich GmbH</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Robin Hein</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>info@uta-gmbh.de</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>06021 / 401922</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>https://www.a-h-a.de/</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>https://uta-gmbh.de/impressum</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>49.988813</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>9.136937</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>node/4420845225</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Mainhof Bäder</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Fritz Loosmann</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>info@maidhof-baeder.de</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>+49 6021 45610 40</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Frohnradstraße 3a</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>63768</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Hösbach</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>https://www.maidhof-baeder.de</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>https://maidhof-baeder.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>50.009602</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>9.215776</t>
+        </is>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>node/6135025622</t>
+        </is>
+      </c>
+      <c r="P127" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Kohl GmbH Heizungsbau</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Kevin Rudolph</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>info@haustechnik-rhein-main.de</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>+49 6021 441570</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Bergstraße 58</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>63814</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Mainaschaff</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>https://haustechnik-rhein-main.de/</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>https://haustechnik-rhein-main.de/kontakt-heizung-klima-sanitaer-aschaffenburg/</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>49.982241</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>9.080075</t>
+        </is>
+      </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>node/9930446355</t>
+        </is>
+      </c>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Hartlieb</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Schlüsseldienst</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr"/>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>info@hartlieb-sicherheit.com</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>+49 6021 75045;+49 5113 12013</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Rohrsängerweg 3</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>63814</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Mainaschaff</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>https://hartlieb-sicherheit.com/</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>https://hartlieb-sicherheit.com/Informationen/Kontakt</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>49.978848</t>
+        </is>
+      </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>9.080648</t>
+        </is>
+      </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>node/9939490586</t>
+        </is>
+      </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Wischfix</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Gebäudereinigung</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Stephan Dietz</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>info@wischfix.com</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>+49 6021 456780</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Paulusstraße 1</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>63741</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>https://www.wischfix.com</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>https://www.wischfix.com/impressum/</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>49.983960</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>9.139706</t>
+        </is>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>node/13196487759</t>
+        </is>
+      </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Bau-Tec</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Bauunternehmen</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Sherif Musliu</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>info@bau-tec.work</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>+49 6021 6296802</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Aschaffenburger Straße 79</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>63773</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Goldbach</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>http://bau-tec.work</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>http://bau-tec.work/imp.html</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>49.997250</t>
+        </is>
+      </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>9.183191</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>node/13260471671</t>
+        </is>
+      </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>EnRo Tiefbau</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Bauunternehmen</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Sherif Musliu</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>info@enro-gmbh.de</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>+49 6181 3044520</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Aschaffenburger Straße 79</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>63773</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Goldbach</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>https://enro-gmbh.de</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>https://enro-gmbh.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>49.997263</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>9.183170</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>node/13260471672</t>
+        </is>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Gallivoda Raumdesign</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Maler / Lackierer</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr"/>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>rene@gallivoda.de</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>+49 171 8230436</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Im Hagen 2</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>63768</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Hösbach</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>https://www.gallivoda-raumdesign.de/</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>https://www.gallivoda-raumdesign.de/kontakt/</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>49.986136</t>
+        </is>
+      </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>9.230502</t>
+        </is>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>node/13314926748</t>
+        </is>
+      </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P108"/>
+  <autoFilter ref="A1:P133"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Nachtlauf: 22 Handwerksbetriebe von Aschaffenburg bis Kleinostheim ergänzen.
Co-authored-by: teamtrack1019 <teamtrack1019@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$P$133</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$P$155</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P133"/>
+  <dimension ref="A1:P155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -10486,8 +10486,1648 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>ELKY</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Eva Kunz</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>info@elkytech.de</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>+49 (0) 6021 12088</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>https://www.elkytech.de/</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>https://www.elkytech.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>49.977703</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>9.152768</t>
+        </is>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>node/2895776521</t>
+        </is>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Malermeister Reißing</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Maler / Lackierer</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr"/>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>info@reissing-malermeister.de</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>+49 6021 624790</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Lorenz-Heim-Straße 19</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>63773</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Goldbach</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>https://reissing-malermeister.de/</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>https://reissing-malermeister.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>50.000920</t>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>9.187104</t>
+        </is>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>node/13564468084</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Uis Gebäudereinigung</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Gebäudereinigung</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Omran Usanmaz</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>info@uis-gebaeudereinigung.de</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>+49 6021 3284261</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr"/>
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>https://www.uis-gebaeudereinigung.de/</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>https://www.uis-gebaeudereinigung.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>49.958517</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>9.117026</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>node/14020358384</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Göhler Schreinerei und Innenausbau</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Schreinerei</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr"/>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>service@schreinerei-goehler.de</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>+49 6021 560048</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Daimlerstraße 4a</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>63768</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Hösbach</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>https://schreinerei-goehler.de/</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>https://schreinerei-goehler.de/</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>50.007737</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>9.216509</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>way/38820531</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>AluTechnik</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Fensterbau</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Jan Horlebein</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>info@alutechnik.com</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Braunstraße 13</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>63741</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>https://www.alutechnik.com/</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>https://alutechnik.com/</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>49.971098</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>9.111835</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>way/94955813</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Philipp Zimlich Präzisionswerkzeuge</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Dipl.-Ing. Ralf Denk</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>info@pza.de</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>bozhin-karaivanov@unsplash.com</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>+49 6021 84740</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Fraunhoferstraße 4</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>63741</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>https://www.pza.de/home.html</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>https://www.pza.de/impressum</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>49.973283</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>9.118503</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>way/94989023</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>SEMCO</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Fensterbau</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr"/>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>info@semcoglas.com</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>info@semcoglas.de; info.aschaffenburg@semcoglas.de; info.sennfeld@semcoglas.de</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>04488 / 840-0</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Dieselstraße 9</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>63741</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>https://www.semcoglas.com/</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>https://www.semcoglas.com/de/kontakt</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>49.984888</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>9.109820</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>way/114724528</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Ernst Aulbach GmbH</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Bauunternehmen</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Alexander Aulbach</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>info@e-aulbach-bau.de</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>06021 424021</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Benzstraße 9</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>https://www.aulbach-bau.de/</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>https://www.aulbach-bau.de/impressum.htm</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>49.983092</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>9.108310</t>
+        </is>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>way/123762956</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Planolith</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Stefan Hein</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>info@planolith.de</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>+49 6021 34 07 0</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Zeppelinstraße 7</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>63741</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>https://www.planolith.de/</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>https://www.planolith.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>49.986261</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>9.108309</t>
+        </is>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>way/123764723</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Hoerig GmbH</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Armin Wengerter</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>info@hoerig-gmbh.de</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>+49 (0) 6021 429310</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Lohmühlstraße 23</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>63741</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>http://www.hoerig-gmbh.de/</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>http://www.hoerig-gmbh.de/html/impressum.html</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>49.990302</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>9.135874</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>way/123910782</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Hartig</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Hartig Beteiligungs</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>info@hartig-germany.com</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>+49 6021 421210</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Lohrweg 6</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>63741</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>https://www.hartig-germany.com/</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>https://hartig-germany.com/impressum/</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>49.990166</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>9.144566</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>way/124149992</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Metallbau Bergmann</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Simon Bergmann</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>info@metallbau-bergmann.de</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>06021/418723</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Magnolienweg 42</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>63741</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>https://www.metallbau-bergmann.de/</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>https://metallbau-bergmann.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>49.969267</t>
+        </is>
+      </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>9.131212</t>
+        </is>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>way/124560701</t>
+        </is>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Schmitt Maschinen</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Doris Gebhardt</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr"/>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>+49(0)6021-45707-0</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Ahornweg 112</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>63741</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>https://www.schmitt-maschinen.com/</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>https://www.schmitt-maschinen.com/de/impressum</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>49.967931</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>9.131808</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>way/124560705</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>nur Geschäftsführer</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Schreinerei Milde</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Zimmerei / Schreinerei</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Günter Milde</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>info@schreinerei-milde.de</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>+49-6028-1560</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Maintalstraße 97</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>63743</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>https://schreinerei-milde.de</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>https://schreinerei-milde.de/impressum</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>49.939960</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>9.129056</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>way/146399389</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Krause Sanitär</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr"/>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>mail@ralfkrause.info</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>+49 6028 992342</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Ruchelnheimstraße 11a</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>https://www.krause-sanitaer.info/</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>https://www.krause-sanitaer.info/kopie-von-impressum</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>49.923170</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>9.154807</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>way/161018339</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Zimmerei Grimm &amp; Wissel</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Bauunternehmen</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Simon Elbert</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>zimmerei@grimm-wissel.de</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>0 60 28 / 99 21 31</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Ruchelnheimstraße 4a</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>63743</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>https://www.grimm-wissel.de</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>https://www.grimm-wissel.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>49.924409</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>9.152285</t>
+        </is>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>way/161019673</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Fenster Stenger GmbH</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Glaserei</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Frank Stenger</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>info@fenster-stenger.de</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>0 60 21 - 62 981 0</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Am Sägewerk 10</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr"/>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>https://www.fenster-stenger.de</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>https://www.fenster-stenger.de/Impressum/DE_index_3009.html</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>49.997047</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>9.188093</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>way/414313535</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Grabmale Karl Hein</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Steinmetz</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Steffen Hein</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>+49 6021 51715</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Aschaffenburger Straße 92</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>63773</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Goldbach</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>http://www.grabmale-hein.de/</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>http://www.grabmale-hein.de/</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>49.997523</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>9.185620</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>way/444751653</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>nur Geschäftsführer</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Horst Roth Stahlbau GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr"/>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>info@stahlbau-roth.de</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>06021 / 45898-0</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Kreuzäcker-Ring 21</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>63814</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Mainaschaff</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>https://www.stahlbau-roth.de/</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>https://stahlbau-roth.de/kontakt/</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>Aschaffenburg</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>49.984588</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>9.101988</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>way/744450726</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Bormann</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Maler / Lackierer</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr"/>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>info@bormann-malerbetrieb.de</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>+49 6021 54196</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Frohnradstraße 18</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>63768</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Hösbach</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>https://www.bormann-malerbetrieb.de/</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>https://www.bormann-malerbetrieb.de/kontakt.html</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>Goldbach</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>50.010209</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>9.222316</t>
+        </is>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>node/13484180685</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Reinfurth Parkett und Bodenbeläge</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Parkettleger</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Heiko Reinfurth</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>info@reinfurth-parkett.de</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr"/>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>06027 124340</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr"/>
+      <c r="H154" t="inlineStr"/>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Kleinostheim</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>https://reinfurth-parkett.de/</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>https://www.reinfurth-parkett.de/impressum.html</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>Kleinostheim</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>50.007405</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>9.061490</t>
+        </is>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>node/12568128955</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>EBS Gebäudereinigung</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Gebäudereinigung</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr"/>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>info@ebs-gebaeudereinigung.de</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>+49 6027 2059895</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Kleinostheim</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>https://www.ebs-gebaeudereinigung.de</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>https://ebs-gebaeudereinigung.de/kontakt/</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>Kleinostheim</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>50.000650</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>9.068487</t>
+        </is>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>node/12684253107</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P133"/>
+  <autoFilter ref="A1:P155"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Nachtlauf: 25 Handwerksbetriebe von Obernburg bis Hanau ergänzen.
Co-authored-by: teamtrack1019 <teamtrack1019@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$P$155</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$P$180</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P155"/>
+  <dimension ref="A1:P180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -12126,8 +12126,1806 @@
         </is>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Fischers NeuArt</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Schreinerei</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr"/>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>info@fischersneuart.de</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr"/>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>+49 6022 8512</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Katharinenstraße 1</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>63785</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>https://www.fischersneuart.de/</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>https://www.fischersneuart.de/ueber-uns/anfahrt-und-kontakt.21e.de.html</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>Obernburg am Main</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>49.839549</t>
+        </is>
+      </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>9.146898</t>
+        </is>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>node/3336463393</t>
+        </is>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>ESH Meisterteam</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Bernd Hilgner</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>info@esh-meisterteam.de</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr"/>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>06027 9905410</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Kleinostheim</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>https://www.esh-meisterteam.de</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>https://www.esh-meisterteam.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>Kleinostheim</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>50.014276</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>9.059689</t>
+        </is>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>node/13566894054</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Elfaisal Elektrotechnik</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr"/>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>hello@elfaisal.de</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>info@elfaisal.de; ka@elfaisal.de</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>+4915124259238</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr"/>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>63801</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Kleinostheim</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>https://elfaisal.de</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>https://elfaisal.de/ueber/impressum/</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>Kleinostheim</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>50.001612</t>
+        </is>
+      </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>9.066161</t>
+        </is>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>node/14093428833</t>
+        </is>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Heinrich Kunkel Straßen- und Tiefbau</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Bauunternehmen</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr"/>
+      <c r="D159" t="inlineStr"/>
+      <c r="E159" t="inlineStr"/>
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr"/>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Kleinostheim</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>https://heinrich-kunkel-tiefbau.de/</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>https://heinrich-kunkel-tiefbau.de/</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>Kleinostheim</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>50.012152</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>9.062593</t>
+        </is>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>way/1450780085</t>
+        </is>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>ohne Kontaktdaten</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Schreinerei Edgar Wissel</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Zimmerei / Schreinerei</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Edgar Wissel</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>info@schreinerei-wissel.de</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr"/>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>+49 6188 4486720</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Industriestraße 5</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>63796</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Kahl am Main</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>https://schreinerei-wissel.de/</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>https://schreinerei-wissel.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>Karlstein am Main</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>50.077297</t>
+        </is>
+      </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>9.013381</t>
+        </is>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>node/2361076335</t>
+        </is>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Grebner Schreinerei</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Zimmerei / Schreinerei</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr"/>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>info@schreinerei-grebner.de</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr"/>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>+49 6188 5292</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Am Kieswerk 14</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>63791</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>Karlstein am Main</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>http://schreinerei-grebner.de</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>http://schreinerei-grebner.de</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>Karlstein am Main</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>50.051619</t>
+        </is>
+      </c>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>9.030947</t>
+        </is>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>node/4293387990</t>
+        </is>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Adler Elektrotechnik GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr"/>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>info@adlerelektro.de</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>info@adlerelectric.com</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>+49 6188 990505</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Kahler Straße 8</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>63791</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Karlstein am Main</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>http://www.adler-elektro.de/</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>https://www.adlerelectric.com</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>Karlstein am Main</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>50.051314</t>
+        </is>
+      </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>9.014205</t>
+        </is>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>node/4293538157</t>
+        </is>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Führer - Heizung &amp; Sanitär</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr"/>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>info@heizungsanitaer-fuehrer.de</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr"/>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>06182 24785</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr"/>
+      <c r="H163" t="inlineStr"/>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Karlstein am Main</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>https://www.heizungsanitaer-fuehrer.de/</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>https://www.heizungsanitaer-fuehrer.de/impressum.html</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>Karlstein am Main</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>50.030278</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>9.026555</t>
+        </is>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>node/4460418544</t>
+        </is>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Koloseus Metallverarbeitung GmbH</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Bernd Koloseus</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>info@koloseus.de</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr"/>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>+49 6188 99530</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr"/>
+      <c r="H164" t="inlineStr"/>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Karlstein am Main</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>https://www.koloseus.de/</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>https://www.koloseus.de/</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>Karlstein am Main</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>50.045437</t>
+        </is>
+      </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>8.996371</t>
+        </is>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>node/5022408922</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Thomas Schielein Heizung Sanitär</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Thomas Schielein</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>info@thomas-schielein.de</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>wodicka@aon.at</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>06023 8124</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Siemensstraße 1</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>63755</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>Alzenau</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>https://www.thomas-schielein.de</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>https://www.thomas-schielein.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>Alzenau</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>50.094184</t>
+        </is>
+      </c>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>9.059591</t>
+        </is>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>node/2361062877</t>
+        </is>
+      </c>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Dachdecker Herd</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Dachdecker</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr"/>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>info@dachdecker-herd.de</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>+49 6023 1333</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Rodenbacher Straße 34</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>63755</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Alzenau</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>http://dachdecker-herd.de/</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>https://dachdecker-herd.de/kontakt/</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>Alzenau</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>50.093122</t>
+        </is>
+      </c>
+      <c r="N166" t="inlineStr">
+        <is>
+          <t>9.061453</t>
+        </is>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>node/4358139271</t>
+        </is>
+      </c>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Glaserei Emmel</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Glaserei</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Michael Emmel</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>info@emmel.de</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr"/>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>06023 9655-0</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Rodenbacher Straße 32</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>63755</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Alzenau</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>https://www.emmel.de/</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>https://www.emmel.de/impressum.html</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>Alzenau</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>50.092699</t>
+        </is>
+      </c>
+      <c r="N167" t="inlineStr">
+        <is>
+          <t>9.061726</t>
+        </is>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>node/4358139272</t>
+        </is>
+      </c>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Schreinerei Amberg</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Schreinerei</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Herrn Stefan Amberg</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>schreinerei.amberg@t-online.de</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr"/>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>+49 6023 5488</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr"/>
+      <c r="H168" t="inlineStr"/>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Alzenau</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>https://schreinerei-amberg.de</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>https://schreinerei-amberg.de/kontakt</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>Alzenau</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>50.105157</t>
+        </is>
+      </c>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>9.104945</t>
+        </is>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>node/12346009945</t>
+        </is>
+      </c>
+      <c r="P168" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Bruder Haustechnik</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr"/>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>info@bruder-haustechnik.de</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>info@sparr.media</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>06182/22436</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr"/>
+      <c r="H169" t="inlineStr"/>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>https://www.bruder-haustechnik.de/</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>https://bruder-haustechnik.de/kontakt</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>50.039018</t>
+        </is>
+      </c>
+      <c r="N169" t="inlineStr">
+        <is>
+          <t>8.969801</t>
+        </is>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>node/3045515618</t>
+        </is>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Stenger Heizung Sanitär Solar GmbH</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Kai Böhm</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>info@stenger-hss.de</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>kundendienst@stenger-hss.de</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>06182 826970</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr"/>
+      <c r="H170" t="inlineStr"/>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>https://www.stenger-hss.de/</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>https://stenger-hss.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>50.044713</t>
+        </is>
+      </c>
+      <c r="N170" t="inlineStr">
+        <is>
+          <t>8.968883</t>
+        </is>
+      </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>node/4354004998</t>
+        </is>
+      </c>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Schreinerei Hock</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Zimmerei / Schreinerei</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Matthias Hock</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr"/>
+      <c r="E171" t="inlineStr"/>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>06182-200121</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr"/>
+      <c r="H171" t="inlineStr"/>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>http://www.schreinerei-seligenstadt.de/</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>https://innenausbau-hock.de/impressum</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>50.050114</t>
+        </is>
+      </c>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>8.970878</t>
+        </is>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>node/4371744820</t>
+        </is>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>nur Geschäftsführer</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Schlosserei Markus Millitzer</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Markus Millitzer</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>info@schlosserei-millitzer-gmbh.de</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr"/>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>+49 6182 28123</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr"/>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>63500</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>http://www.schlosserei-millitzer-gmbh.de/</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>http://www.schlosserei-millitzer-gmbh.de/common/info/impressum.html</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>50.045405</t>
+        </is>
+      </c>
+      <c r="N172" t="inlineStr">
+        <is>
+          <t>8.973665</t>
+        </is>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>node/5000124367</t>
+        </is>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Bühring GmbH</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Karsten Bühring</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>info@buehring-gmbh.com</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr"/>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>0 61 82 / 54 62</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr"/>
+      <c r="H173" t="inlineStr"/>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>http://buehring-gmbh.com/</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>http://buehring-gmbh.com/impressum.html</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>50.074317</t>
+        </is>
+      </c>
+      <c r="N173" t="inlineStr">
+        <is>
+          <t>8.966867</t>
+        </is>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>node/6431536082</t>
+        </is>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>RohrStar Rohrreinigung</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr"/>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>zentrale@rohrstar.de</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>offenbach@rohrstar.de; kahl@rohrstar.de; jacob@rohrstar.de</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>+49 6182 787787</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr"/>
+      <c r="H174" t="inlineStr"/>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>https://rohrstar.de/rohrsanierung-hainburg</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>https://rohrstar.de/impressum</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>50.065905</t>
+        </is>
+      </c>
+      <c r="N174" t="inlineStr">
+        <is>
+          <t>8.967129</t>
+        </is>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>node/6432220264</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>PURCRAFT GmbH</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Daniel Bücking</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>info@purcraft.de</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr"/>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>+49 6182 772653-0</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr"/>
+      <c r="H175" t="inlineStr"/>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>https://purcraft.de</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>https://purcraft.de/imprint/</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>50.036651</t>
+        </is>
+      </c>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>8.960091</t>
+        </is>
+      </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>node/7026546597</t>
+        </is>
+      </c>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>esatek</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Ralf Stenger</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>anfrage@esatek.de</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>solaranfrage@esatek.de</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>+49-6182-829047</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr"/>
+      <c r="H176" t="inlineStr"/>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>https://www.esatek.de</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>https://www.esatek.de/impressum.html</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>50.052560</t>
+        </is>
+      </c>
+      <c r="N176" t="inlineStr">
+        <is>
+          <t>8.968183</t>
+        </is>
+      </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>node/14019983829</t>
+        </is>
+      </c>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Meister Winter</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Michael Winter</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr"/>
+      <c r="E177" t="inlineStr"/>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>+49(0)6182/7701600</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr"/>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>https://www.meisterwinter.de</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>https://www.meisterwinter.de/about/</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>Seligenstadt</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>50.041016</t>
+        </is>
+      </c>
+      <c r="N177" t="inlineStr">
+        <is>
+          <t>8.972558</t>
+        </is>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>node/14022593810</t>
+        </is>
+      </c>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>nur Geschäftsführer</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Steinmetz Detzner</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Steinmetz</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Martina Detzner</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>anfrage@steinmetz-detzner.com</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>steinmetz-detzner@t-online.de</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>06186 1734</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="inlineStr"/>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>Hainburg</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>https://www.steinmetz-detzner.com</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>https://www.steinmetz-detzner.com/</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>Hainburg</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>50.085854</t>
+        </is>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>8.961948</t>
+        </is>
+      </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>node/14006783293</t>
+        </is>
+      </c>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Kälte-Pietz</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Markus Freund</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>info@kaelte-pietz.de</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr"/>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>06023 96800 200</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr"/>
+      <c r="H179" t="inlineStr"/>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>Hainburg</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>https://kaelte-pietz.de</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>https://kaelte-pietz.de/</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>Hainburg</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>50.083848</t>
+        </is>
+      </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>8.966343</t>
+        </is>
+      </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>node/14006800358</t>
+        </is>
+      </c>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>maba! Maler- und Ausbau- werkstätten GmbH</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Maler / Lackierer</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Hannes Brandtstäter</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>service@maba-gmbh.de</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>kuhnle@maba-gmbh.de</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>+49 6181 300330</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr"/>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>https://maba-gmbh.de</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>https://maba-gmbh.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>50.151977</t>
+        </is>
+      </c>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>8.939128</t>
+        </is>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>node/3812451242</t>
+        </is>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P155"/>
+  <autoFilter ref="A1:P180"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Nachtlauf: 21 Handwerksbetriebe von Hanau bis Maintal ergänzen.
Co-authored-by: teamtrack1019 <teamtrack1019@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$P$180</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$P$201</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P180"/>
+  <dimension ref="A1:P201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -13924,8 +13924,1566 @@
         </is>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Schlosserei Kürschner</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Stephan Kürschner</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>info@kuerschner-kg.de</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr"/>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>+49 6181 79709</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Hauptstraße 73</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>63486</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>Bruchköbel</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>https://www.xn--krschner-kg-thb.de/index.html</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>https://www.xn--krschner-kg-thb.de/impressum-kuerschner-kg.html</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>50.178648</t>
+        </is>
+      </c>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>8.922186</t>
+        </is>
+      </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>node/7868134390</t>
+        </is>
+      </c>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>E.T.S. Elektro Technik Schmidt</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr"/>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>info@ets-schmidt.de</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr"/>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>+49 6181 3077866</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Hauptstraße 93</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>63486</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>Bruchköbel</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>https://www.ets-schmidt.de/</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>https://www.ets-schmidt.de/kontakt/</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>50.179173</t>
+        </is>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>8.924444</t>
+        </is>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>node/7868134409</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Oetjen GmbH</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Sven Oetjen</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>info@oetjen-gmbh.de</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr"/>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>+49 6181 575430</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Limesstraße 1A</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>63486</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>Bruchköbel</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>https://www.oetjen-gmbh.de/</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>https://www.oetjen-gmbh.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>50.180857</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>8.910734</t>
+        </is>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>node/9223503914</t>
+        </is>
+      </c>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Emmel Malerdesign</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Maler / Lackierer</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr"/>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>info@emmel-malerdesign.de</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>mail@emmel-malerdesign.de</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>+49 6181 71293</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr"/>
+      <c r="H184" t="inlineStr"/>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>https://www.emmel-malerdesign.de/</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>https://www.emmel-malerdesign.de/kontakt/</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>50.180477</t>
+        </is>
+      </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>8.912619</t>
+        </is>
+      </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>node/9223503916</t>
+        </is>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>AMP Altbausanierung</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Bauunternehmen</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Marco Palacios</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>info@amp-altbausanierung.de</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr"/>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>+49 6181 9060640</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Philipp-Reis-Straße 10</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>63486</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>Bruchköbel</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>http://www.amp-altbausanierung.de</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>http://www.amp-altbausanierung.de/impressum.html</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>50.183244</t>
+        </is>
+      </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>8.914327</t>
+        </is>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>node/9223510850</t>
+        </is>
+      </c>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Schreinerei Ertelt</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Schreinerei</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr"/>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>info@schreinerei-ertelt.de</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>mail@architektur-denkmalpflege.net; mail@stefanmarquardt.de</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>+49 6181 72118</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Friedberger Landstraße 8</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>63486</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>Bruchköbel</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>https://www.schreinerei-ertelt.de</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>https://www.schreinerei-ertelt.de/kontakt</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>50.182892</t>
+        </is>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>8.913509</t>
+        </is>
+      </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>node/9223510913</t>
+        </is>
+      </c>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Peter Viel</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Jürgen Viel</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>info@viel-online.de</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr"/>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>+49 6183 3935</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr"/>
+      <c r="H187" t="inlineStr"/>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>https://www.viel-online.de/</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>https://www.viel-online.de/kontakt/</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>50.161104</t>
+        </is>
+      </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>8.979599</t>
+        </is>
+      </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>node/10838947358</t>
+        </is>
+      </c>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>artbau</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Dieter Dittmar</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>info@artbau-gmbh.de</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>info@artbau-projekt.de; info@artbau-technik.de</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>+49 6181 364677 0</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr"/>
+      <c r="H188" t="inlineStr"/>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>https://www.artbau-gmbh.de/</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>https://www.artbau-gmbh.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>50.183673</t>
+        </is>
+      </c>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>8.915524</t>
+        </is>
+      </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>node/11157558877</t>
+        </is>
+      </c>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Heinrich Struve Sanitär- und Heizungstechnik GmbH</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Dipl.-Ing. Ramazan Cayir</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>info@struve-hanau.de</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr"/>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>+49618182077</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr"/>
+      <c r="H189" t="inlineStr"/>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>https://struve-hanau.de/</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>https://struve-hanau.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>50.146975</t>
+        </is>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>8.908182</t>
+        </is>
+      </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>node/11898490671</t>
+        </is>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Elektro Heinrich Seib GmbH</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Christian Seib</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>c.seib@elektro-seib.de</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>mail@universalschlichtungsstelle.de</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>+49 6181 980810</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Bruchköbeler Landstraße 11</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>63452</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>http://elektro-seib.de</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>https://www.elektro-seib.de/kontakt/impressum</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>50.141025</t>
+        </is>
+      </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>8.911255</t>
+        </is>
+      </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>node/11898600070</t>
+        </is>
+      </c>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Elektrobau Kraft</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Elektriker</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Ralf Kraft</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>info@kraft-elektrobau.de</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr"/>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>+49 6181 97200</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Am Germanenring 36</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>63486</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>Bruchköbel</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>https://kraft-elektrobau.de</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>https://www.kraft-elektrobau.de/impressum.html</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>50.174572</t>
+        </is>
+      </c>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>8.909283</t>
+        </is>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>node/11901261105</t>
+        </is>
+      </c>
+      <c r="P191" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Abfluss Schäfer</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr"/>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>info@abfluss-schaefer-gmbh.de</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>service@ffm.media</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>+49 6183 9284200</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr"/>
+      <c r="H192" t="inlineStr"/>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>https://www.abfluss-schaefer-gmbh.de/</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>https://www.abfluss-schaefer-gmbh.de/kontakt/</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>50.162638</t>
+        </is>
+      </c>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>8.954813</t>
+        </is>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>node/12506312696</t>
+        </is>
+      </c>
+      <c r="P192" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Glaserei Zeiler GmbH</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Glaserei</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Uwe Zeiler</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>info@glaserei-zeiler.de</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>info@glasereizeiler.de</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>+49 6181 4238592</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Philipp-Reis-Straße 13</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>63486</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Bruchköbel</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>https://glaserei-zeiler.de/</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>https://www.glaserei-zeiler.de/impressum</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>50.184066</t>
+        </is>
+      </c>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>8.915973</t>
+        </is>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>way/197755177</t>
+        </is>
+      </c>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Heck GmbH</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr"/>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>info@heck-gmbh.de</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>info@ieq-systems-shk.de; ofke@mn.dcegibhh</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>+49 6181 21462</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Hopfenstraße 8</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>63454</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>https://www.heck-gmbh.de/</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>https://www.heck-gmbh.de/unternehmen/proweb-advanced/kontakt</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>50.132700</t>
+        </is>
+      </c>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>8.896876</t>
+        </is>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>way/234018329</t>
+        </is>
+      </c>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Christian Schultheis Bedachungen</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Dachdecker</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr"/>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>info@schultheis-dach.de</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>info@kh-hanau.de; gewerbeamt@hanau.de</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>06181 / 9939-0</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr"/>
+      <c r="H195" t="inlineStr"/>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>https://www.schultheis-dach.de/</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>https://www.schultheis-dach.de/kontakt.html</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>Hanau</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>50.173828</t>
+        </is>
+      </c>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>8.910231</t>
+        </is>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>way/1385034203</t>
+        </is>
+      </c>
+      <c r="P195" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Steinmetzbetrieb Möller</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Steinmetz</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr"/>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>mail@steinmetz-moeller.de</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr"/>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>06181/71355</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Pfingstweidstraße 3</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>63486</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>Bruchköbel</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>https://www.steinmetz-moeller.de/</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>https://www.steinmetz-moeller.de/</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>Bruchköbel</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>50.198122</t>
+        </is>
+      </c>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>8.906399</t>
+        </is>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>node/10840423733</t>
+        </is>
+      </c>
+      <c r="P196" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Alfred Kaut GmbH &amp; Co.</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr"/>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>info@kaut.de</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>mail@kaut.de; office@kaut.de; kg.jobs@kaut.de</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>+49 6109 69680</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr"/>
+      <c r="H197" t="inlineStr"/>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Maintal</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>https://www.kaut.de</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>https://www.kaut.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>Maintal</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>50.141951</t>
+        </is>
+      </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>8.809462</t>
+        </is>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>node/4121082518</t>
+        </is>
+      </c>
+      <c r="P197" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Emerson Climate Technologies GmbH</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr"/>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>data.privacy@copeland.com</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>legal@copeland.com</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>+49 6109 60590</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr"/>
+      <c r="H198" t="inlineStr"/>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Maintal</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>https://www.ecopeland.com/</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>https://www.copeland.com/en-us</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>Maintal</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>50.141969</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>8.809057</t>
+        </is>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>node/4121082519</t>
+        </is>
+      </c>
+      <c r="P198" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Die Steinwerkstatt Stefan Schneider</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Steinmetz</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Stefan Schneider</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>info@steinwerkstatt-schneider.de</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>info@hwk-rhein-main.de</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>069 865661</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr"/>
+      <c r="H199" t="inlineStr"/>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Maintal</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>https://www.steinwerkstatt-schneider.de/</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>https://www.steinwerkstatt-schneider.de/impressum</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>Maintal</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>50.113423</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>8.808216</t>
+        </is>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>node/9065688392</t>
+        </is>
+      </c>
+      <c r="P199" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Schneider Grabmale</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Steinmetz</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr"/>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>info@schneider-grabmale.com</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr"/>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>069 86 2002</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr"/>
+      <c r="H200" t="inlineStr"/>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Maintal</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>https://schneider-grabmale.com/</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>https://www.schneider-grabmale.com/kontakt</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>Maintal</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>50.115762</t>
+        </is>
+      </c>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>8.809838</t>
+        </is>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>node/9065763541</t>
+        </is>
+      </c>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Böhm Schreinerei Glaserei</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Zimmerei / Schreinerei</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr"/>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>info@boehm-schreinerei-glaserei.de</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr"/>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>+49 6108 7969960</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Zimmerstraße 51</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>63165</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Mühlheim am Main</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>http://dirk-winkler.com/</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>http://dirk-winkler.com/</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>Maintal</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>50.120037</t>
+        </is>
+      </c>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>8.834426</t>
+        </is>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>node/13701669417</t>
+        </is>
+      </c>
+      <c r="P201" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P180"/>
+  <autoFilter ref="A1:P201"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Nachtlauf: 19 Handwerksbetriebe von Maintal bis Frankfurt ergänzen.
Co-authored-by: teamtrack1019 <teamtrack1019@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$P$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads'!$A$1:$P$220</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P201"/>
+  <dimension ref="A1:P220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -541,13 +541,11 @@
           <t>Motorrad</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>wuerzburg@polo-motorrad.com</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>+49 931 2700042</t>
@@ -615,7 +613,6 @@
           <t>Bäckerei</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>info@koehlers-vollkornbaeckerei.de</t>
@@ -785,7 +782,6 @@
           <t>info@velo-momber.de</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>+49 931 12627</t>
@@ -863,7 +859,6 @@
           <t>info@baeckerei-schiffer.com</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>0931 53271</t>
@@ -941,7 +936,6 @@
           <t>info@bb-roesner-backstube.de</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>+49 931 6192082</t>
@@ -1091,13 +1085,11 @@
           <t>Dienstleister (cafe)</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>mehlbox@baecker-roth.de</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>+49 931 64149</t>
@@ -1165,13 +1157,11 @@
           <t>Bäckerei</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>info@backkunst.de</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>+49 931 3297989</t>
@@ -1249,8 +1239,6 @@
           <t>metzgermeister.holz@gmail.com</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>Erlabrunner Straße 4</t>
@@ -1313,7 +1301,6 @@
           <t>Metzgerei</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>info@metzgerei-flach.de</t>
@@ -1483,7 +1470,6 @@
           <t>info@bb-roesner-backstube.de</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>+49 931 4046746</t>
@@ -1551,7 +1537,6 @@
           <t>Friseur</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>info@hairstyle-friseur.de</t>
@@ -1721,7 +1706,6 @@
           <t>kontakt@maxlbaeck.de</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>+49 931 413004</t>
@@ -1799,14 +1783,11 @@
           <t>info@tatenwerk.social</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>+49 931 7960514</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -1951,7 +1932,6 @@
           <t>verkauf@fahrradprofis.info</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>+49 931 12338</t>
@@ -2183,9 +2163,6 @@
           <t>Mobilfunk</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>+49 931 30418645</t>
@@ -2253,13 +2230,11 @@
           <t>Schmuck</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>info@juwelier-endres.de</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>+49 931 52735</t>
@@ -2419,7 +2394,6 @@
           <t>info@bb-roesner-backstube.de</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>+49 931 4606111</t>
@@ -2497,7 +2471,6 @@
           <t>info@bb-roesner-backstube.de</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>+49 931 3040398</t>
@@ -2657,7 +2630,6 @@
           <t>info@schmucklaedele.de</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>+49 931 58299</t>
@@ -2725,20 +2697,16 @@
           <t>Optiker</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>info@brillenstudio-am-markt.de</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>+49 931 13666</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -2791,13 +2759,11 @@
           <t>Fahrrad</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>info@bikestore-wuerzburg.de</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>+49 931 77039</t>
@@ -3049,8 +3015,6 @@
           <t>+49 931 3548855</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -3185,13 +3149,11 @@
           <t>Eisenwaren</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>schraubensepp@email.de</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>+49 931 4045353</t>
@@ -3269,7 +3231,6 @@
           <t>info@rohrwasser-issing.de</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>+49 931 3535200</t>
@@ -3347,7 +3308,6 @@
           <t>info@auto-kilian.de</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>+49 931 2500600</t>
@@ -3415,13 +3375,11 @@
           <t>Computer</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
           <t>info@pcsweb.de</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>+49 931 2878071</t>
@@ -3591,8 +3549,6 @@
           <t>+49 931 880753-0</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -3645,7 +3601,6 @@
           <t>Metallbau</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
           <t>info@roeder-metallbau.de</t>
@@ -3661,8 +3616,6 @@
           <t>0931 / 93263</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -3715,13 +3668,11 @@
           <t>Maler / Lackierer</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
           <t>ferschmalt@ferschmalt.de</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>+49 9302 1223</t>
@@ -3799,7 +3750,6 @@
           <t>fensterbau-zinnhobel@t-online.de</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>+49 931 9917360</t>
@@ -3867,7 +3817,6 @@
           <t>Sanitär / Heizung</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
           <t>info@ziegler-shk.de</t>
@@ -3955,14 +3904,11 @@
           <t>info@conzept-bad.de</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>0931 - 20 53 53 0</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -4025,7 +3971,6 @@
           <t>info@hilpert-heizung.de</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>+49 931 79780 0</t>
@@ -4103,7 +4048,6 @@
           <t>info@pixis.de</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>+49 931 70560-0</t>
@@ -4171,19 +4115,16 @@
           <t>Schlüsseldienst</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
           <t>info@schluessel-goetz.de</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>+49 931 53525</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>97070</t>
@@ -4343,8 +4284,6 @@
           <t>+49 9365 80840</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -4397,20 +4336,16 @@
           <t>Sanitär / Heizung</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
           <t>office@weber-martin.de</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>0931 / 7840947</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -4555,7 +4490,6 @@
           <t>info@stein-welten.com</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>+49 931 20029 0</t>
@@ -4633,7 +4567,6 @@
           <t>info@heckelmann-kirchner.de</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>0931 / 27 049 700</t>
@@ -4701,9 +4634,6 @@
           <t>Zimmerei / Schreinerei</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>+49 931 8807997</t>
@@ -4781,7 +4711,6 @@
           <t>info@porzner.com</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>+49 931 461234</t>
@@ -4792,7 +4721,6 @@
           <t>Hauptstraße 130</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -4855,7 +4783,6 @@
           <t>info@moritz-wuerzburg.de</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>+49 931 797810</t>
@@ -4923,20 +4850,16 @@
           <t>Fensterbau</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
           <t>info@fenster-neumueller.de</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>+49 931 30196635</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -4989,20 +4912,16 @@
           <t>Schreinerei</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
           <t>info@maintisch.de</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>+49 1512 0101070</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -5065,14 +4984,11 @@
           <t>info@walter-breunig.de</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>+49 931 80996910</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -5125,13 +5041,11 @@
           <t>Elektriker</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
           <t>info@hesselbarth-get.de</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>+49 931 304296 0</t>
@@ -5209,14 +5123,11 @@
           <t>info@zimmerei-geiger.de</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>+49 931 45249800</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -5279,14 +5190,11 @@
           <t>info@flammersberger.com</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>+49 931 970090</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -5359,8 +5267,6 @@
           <t>0931 / 94698</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -5423,14 +5329,11 @@
           <t>info@wuerzburger-pflasterbau.de</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>+49 931 980690</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -5483,12 +5386,6 @@
           <t>Metallbau</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -5551,7 +5448,6 @@
           <t>info@glaserei-nagel.de</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>0931 - 26 43 4</t>
@@ -5629,7 +5525,6 @@
           <t>info@schumann-kreativwerkstatt.de</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>+49 931 78023 516</t>
@@ -5697,20 +5592,16 @@
           <t>Fliesenleger</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
           <t>info@fliesenlazar.de</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>+49 931 35820198</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr">
         <is>
           <t>Würzburg</t>
@@ -5763,13 +5654,11 @@
           <t>Gebäudereinigung</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
           <t>ruegamer.gebaeudeservice@gmx.net</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>+49 931 53166</t>
@@ -5847,13 +5736,11 @@
           <t>info@viessmann-climatesolutions.com</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>+4993161550</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>97076</t>
@@ -5911,13 +5798,11 @@
           <t>Heizung / Klima</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
           <t>info@kimmel-gmbh.de</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>+49 931 99135900</t>
@@ -5995,7 +5880,6 @@
           <t>info@fmeder.de</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>+49 931 42539</t>
@@ -6073,7 +5957,6 @@
           <t>info@beck-elektrotechnik.de</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>+49 931 20050</t>
@@ -6305,7 +6188,6 @@
           <t>Steinmetz</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr">
         <is>
           <t>info@steinwerk-haas.de</t>
@@ -6475,7 +6357,6 @@
           <t>mw@schreinerei-walk.de</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>+49 9306 1376</t>
@@ -6553,7 +6434,6 @@
           <t>service@rms-metalwork.de</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
           <t>+49 9306 8599</t>
@@ -6621,7 +6501,6 @@
           <t>Glaserei</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr">
         <is>
           <t>info@deutschesglas.de</t>
@@ -6709,7 +6588,6 @@
           <t>info@bauunternehmung-blank.de</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
           <t>+49 9369 1666</t>
@@ -6782,8 +6660,6 @@
           <t>Christoph Ruhland</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
           <t>09342- 935 -</t>
@@ -6943,7 +6819,6 @@
           <t>info@felix-bauer.com</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
           <t>+49 9371 948939 0</t>
@@ -7016,8 +6891,6 @@
           <t>Achim Hawel</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
           <t>+49 9371 8422</t>
@@ -7095,7 +6968,6 @@
           <t>info@maler-riegel.de</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
           <t>+49 9371 1281</t>
@@ -7183,8 +7055,6 @@
           <t>+49 9371 67764</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
           <t>Miltenberg</t>
@@ -7237,20 +7107,16 @@
           <t>Metallbau</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
           <t>peter@dietz-metallbau.de</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
           <t>+49 171 1719889</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr"/>
       <c r="I90" t="inlineStr">
         <is>
           <t>Miltenberg</t>
@@ -7303,13 +7169,11 @@
           <t>Elektriker</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr">
         <is>
           <t>franz-zoeller@fz-elektro.de</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
           <t>+49 9371 682 82</t>
@@ -7387,14 +7251,11 @@
           <t>info@cs-mil.de</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>+49 9371 657 79</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr"/>
       <c r="I92" t="inlineStr">
         <is>
           <t>Miltenberg</t>
@@ -7447,20 +7308,16 @@
           <t>Elektriker</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
           <t>firma@ta-elektrotechnik.de</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>+49 9371 601 7125</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
           <t>Miltenberg</t>
@@ -7605,7 +7462,6 @@
           <t>info@schneider-raum.de</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
           <t>09371/94730-0</t>
@@ -7616,7 +7472,6 @@
           <t>Im Bruch 1</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
           <t>Miltenberg</t>
@@ -7684,13 +7539,11 @@
           <t>anfrage@main-pv.de</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
           <t>Lassallestraße 7</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
       <c r="I96" t="inlineStr">
         <is>
           <t>Miltenberg</t>
@@ -7743,7 +7596,6 @@
           <t>Metallbau</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr">
         <is>
           <t>info@breitenbach-metall.de</t>
@@ -7841,8 +7693,6 @@
           <t>+49 9372 923856</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr"/>
       <c r="I98" t="inlineStr">
         <is>
           <t>Miltenberg</t>
@@ -7905,7 +7755,6 @@
           <t>info@heim-steintechnik.de</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
           <t>09371 668010</t>
@@ -7983,7 +7832,6 @@
           <t>info@hefner-boden.de</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
           <t>0 93 71 - 94 99 480</t>
@@ -8051,13 +7899,11 @@
           <t>Schreinerei</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
           <t>info@schreiner-fichtl.de</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
           <t>+49 6022 2086113</t>
@@ -8135,7 +7981,6 @@
           <t>info@raku-gmbh.de</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>+49 6022 9073</t>
@@ -8213,7 +8058,6 @@
           <t>info@rehm-trockenbau.de</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
           <t>+49 6022 5072011</t>
@@ -8281,13 +8125,11 @@
           <t>Fensterbau</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr"/>
       <c r="D104" t="inlineStr">
         <is>
           <t>pwagner@wagner-bausysteme.com</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
           <t>+49 6022 5067444</t>
@@ -8365,7 +8207,6 @@
           <t>info@ms-elektro-technik.de</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
           <t>+49 6022 710100</t>
@@ -8376,7 +8217,6 @@
           <t>Im Höning 20</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr">
         <is>
           <t>Obernburg am Main</t>
@@ -8429,9 +8269,6 @@
           <t>Elektriker</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr"/>
-      <c r="D106" t="inlineStr"/>
-      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
           <t>+49 9372 940239</t>
@@ -8509,7 +8346,6 @@
           <t>info@kelpetin.eu</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>+4915141912358</t>
@@ -8587,14 +8423,11 @@
           <t>info@fath-bau.com</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
           <t>+49 170 9129431</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
       <c r="I108" t="inlineStr">
         <is>
           <t>Obernburg am Main</t>
@@ -8657,7 +8490,6 @@
           <t>buero@zwissler.eu</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
           <t>+49 9371 3909</t>
@@ -8725,13 +8557,11 @@
           <t>Elektriker</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr"/>
       <c r="D110" t="inlineStr">
         <is>
           <t>kontakt@tw-elektrotechnik.com</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
           <t>+49 6022 6524389</t>
@@ -8809,7 +8639,6 @@
           <t>info@faerbergmbh.de</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
           <t>06022/71094-0 -</t>
@@ -8877,13 +8706,11 @@
           <t>Zimmerei / Schreinerei</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr"/>
       <c r="D112" t="inlineStr">
         <is>
           <t>info@zimmerei-boneberger.de</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>+49 6022 2233</t>
@@ -8961,7 +8788,6 @@
           <t>info@malerforum.com</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
           <t>+49 6022 7093330</t>
@@ -9034,8 +8860,6 @@
           <t>Julia Brenner</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr"/>
-      <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
           <t>+49 6022 2631-0</t>
@@ -9113,14 +8937,11 @@
           <t>info@loewe-fenster.de</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
           <t>+49 6022 6630-0</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
-      <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
           <t>Obernburg am Main</t>
@@ -9173,13 +8994,11 @@
           <t>Elektriker</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr">
         <is>
           <t>info@roth-elektrotechnik.com</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
           <t>+49 6022 2655880</t>
@@ -9190,7 +9009,6 @@
           <t>Grundtalring 45</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
       <c r="I116" t="inlineStr">
         <is>
           <t>Obernburg am Main</t>
@@ -9243,7 +9061,6 @@
           <t>Schreinerei</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr"/>
       <c r="D117" t="inlineStr">
         <is>
           <t>info@schreinereiml.com</t>
@@ -9331,14 +9148,11 @@
           <t>info@schreinerei-hammerbacher.de</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
           <t>+49 (0) 6021 / 2 25 96</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr"/>
-      <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr">
         <is>
           <t>Aschaffenburg</t>
@@ -9391,20 +9205,16 @@
           <t>Steinmetz</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr">
         <is>
           <t>info@steinwerk-hirte.de</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
           <t>06021 929485</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr"/>
-      <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr">
         <is>
           <t>Aschaffenburg</t>
@@ -9549,14 +9359,11 @@
           <t>info@ulltech-ag.de</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr">
         <is>
           <t>06021-386530</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
-      <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
           <t>Aschaffenburg</t>
@@ -9619,14 +9426,11 @@
           <t>info@glasstudio-bergmann.de</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr">
         <is>
           <t>+49 6021 28484</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
-      <c r="H122" t="inlineStr"/>
       <c r="I122" t="inlineStr">
         <is>
           <t>Aschaffenburg</t>
@@ -9689,14 +9493,11 @@
           <t>info@benedict-gmbh.de</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
           <t>+49 (0)6021</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr"/>
-      <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
           <t>Aschaffenburg</t>
@@ -9759,14 +9560,11 @@
           <t>kontakt@gkk.net</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
           <t>+49-6021-34940</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr"/>
-      <c r="H124" t="inlineStr"/>
       <c r="I124" t="inlineStr">
         <is>
           <t>Aschaffenburg</t>
@@ -9819,7 +9617,6 @@
           <t>Elektriker</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr">
         <is>
           <t>mail@universalschlichtungsstelle.de</t>
@@ -9835,8 +9632,6 @@
           <t>06021/5851666</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr"/>
-      <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr">
         <is>
           <t>Aschaffenburg</t>
@@ -9899,14 +9694,11 @@
           <t>info@uta-gmbh.de</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr">
         <is>
           <t>06021 / 401922</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr"/>
-      <c r="H126" t="inlineStr"/>
       <c r="I126" t="inlineStr">
         <is>
           <t>Aschaffenburg</t>
@@ -9969,7 +9761,6 @@
           <t>info@maidhof-baeder.de</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr">
         <is>
           <t>+49 6021 45610 40</t>
@@ -10047,7 +9838,6 @@
           <t>info@haustechnik-rhein-main.de</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr">
         <is>
           <t>+49 6021 441570</t>
@@ -10115,13 +9905,11 @@
           <t>Schlüsseldienst</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr"/>
       <c r="D129" t="inlineStr">
         <is>
           <t>info@hartlieb-sicherheit.com</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
           <t>+49 6021 75045;+49 5113 12013</t>
@@ -10199,7 +9987,6 @@
           <t>info@wischfix.com</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
           <t>+49 6021 456780</t>
@@ -10277,7 +10064,6 @@
           <t>info@bau-tec.work</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
           <t>+49 6021 6296802</t>
@@ -10355,7 +10141,6 @@
           <t>info@enro-gmbh.de</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
           <t>+49 6181 3044520</t>
@@ -10423,13 +10208,11 @@
           <t>Maler / Lackierer</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr">
         <is>
           <t>rene@gallivoda.de</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr">
         <is>
           <t>+49 171 8230436</t>
@@ -10507,14 +10290,11 @@
           <t>info@elkytech.de</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
         <is>
           <t>+49 (0) 6021 12088</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr"/>
-      <c r="H134" t="inlineStr"/>
       <c r="I134" t="inlineStr">
         <is>
           <t>Aschaffenburg</t>
@@ -10567,13 +10347,11 @@
           <t>Maler / Lackierer</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr">
         <is>
           <t>info@reissing-malermeister.de</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr">
         <is>
           <t>+49 6021 624790</t>
@@ -10651,14 +10429,11 @@
           <t>info@uis-gebaeudereinigung.de</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
           <t>+49 6021 3284261</t>
         </is>
       </c>
-      <c r="G136" t="inlineStr"/>
-      <c r="H136" t="inlineStr"/>
       <c r="I136" t="inlineStr">
         <is>
           <t>Aschaffenburg</t>
@@ -10711,13 +10486,11 @@
           <t>Schreinerei</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr">
         <is>
           <t>service@schreinerei-goehler.de</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr">
         <is>
           <t>+49 6021 560048</t>
@@ -10795,8 +10568,6 @@
           <t>info@alutechnik.com</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
-      <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
           <t>Braunstraße 13</t>
@@ -10941,7 +10712,6 @@
           <t>Fensterbau</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr">
         <is>
           <t>info@semcoglas.com</t>
@@ -11029,7 +10799,6 @@
           <t>info@e-aulbach-bau.de</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr">
         <is>
           <t>06021 424021</t>
@@ -11040,7 +10809,6 @@
           <t>Benzstraße 9</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr"/>
       <c r="I141" t="inlineStr">
         <is>
           <t>Aschaffenburg</t>
@@ -11103,7 +10871,6 @@
           <t>info@planolith.de</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
           <t>+49 6021 34 07 0</t>
@@ -11181,7 +10948,6 @@
           <t>info@hoerig-gmbh.de</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
           <t>+49 (0) 6021 429310</t>
@@ -11259,7 +11025,6 @@
           <t>info@hartig-germany.com</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr"/>
       <c r="F144" t="inlineStr">
         <is>
           <t>+49 6021 421210</t>
@@ -11337,7 +11102,6 @@
           <t>info@metallbau-bergmann.de</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr"/>
       <c r="F145" t="inlineStr">
         <is>
           <t>06021/418723</t>
@@ -11410,8 +11174,6 @@
           <t>Doris Gebhardt</t>
         </is>
       </c>
-      <c r="D146" t="inlineStr"/>
-      <c r="E146" t="inlineStr"/>
       <c r="F146" t="inlineStr">
         <is>
           <t>+49(0)6021-45707-0</t>
@@ -11489,7 +11251,6 @@
           <t>info@schreinerei-milde.de</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr">
         <is>
           <t>+49-6028-1560</t>
@@ -11557,13 +11318,11 @@
           <t>Sanitär / Heizung</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr"/>
       <c r="D148" t="inlineStr">
         <is>
           <t>mail@ralfkrause.info</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr">
         <is>
           <t>+49 6028 992342</t>
@@ -11574,7 +11333,6 @@
           <t>Ruchelnheimstraße 11a</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr"/>
       <c r="I148" t="inlineStr">
         <is>
           <t>Aschaffenburg</t>
@@ -11637,7 +11395,6 @@
           <t>zimmerei@grimm-wissel.de</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr">
         <is>
           <t>0 60 28 / 99 21 31</t>
@@ -11715,7 +11472,6 @@
           <t>info@fenster-stenger.de</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr">
         <is>
           <t>0 60 21 - 62 981 0</t>
@@ -11726,7 +11482,6 @@
           <t>Am Sägewerk 10</t>
         </is>
       </c>
-      <c r="H150" t="inlineStr"/>
       <c r="I150" t="inlineStr">
         <is>
           <t>Aschaffenburg</t>
@@ -11784,8 +11539,6 @@
           <t>Steffen Hein</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr"/>
-      <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr">
         <is>
           <t>+49 6021 51715</t>
@@ -11853,13 +11606,11 @@
           <t>Metallbau</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr"/>
       <c r="D152" t="inlineStr">
         <is>
           <t>info@stahlbau-roth.de</t>
         </is>
       </c>
-      <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr">
         <is>
           <t>06021 / 45898-0</t>
@@ -11927,13 +11678,11 @@
           <t>Maler / Lackierer</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr"/>
       <c r="D153" t="inlineStr">
         <is>
           <t>info@bormann-malerbetrieb.de</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr">
         <is>
           <t>+49 6021 54196</t>
@@ -12011,14 +11760,11 @@
           <t>info@reinfurth-parkett.de</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr">
         <is>
           <t>06027 124340</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr"/>
-      <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr">
         <is>
           <t>Kleinostheim</t>
@@ -12071,20 +11817,16 @@
           <t>Gebäudereinigung</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr">
         <is>
           <t>info@ebs-gebaeudereinigung.de</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr"/>
       <c r="F155" t="inlineStr">
         <is>
           <t>+49 6027 2059895</t>
         </is>
       </c>
-      <c r="G155" t="inlineStr"/>
-      <c r="H155" t="inlineStr"/>
       <c r="I155" t="inlineStr">
         <is>
           <t>Kleinostheim</t>
@@ -12137,13 +11879,11 @@
           <t>Schreinerei</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr"/>
       <c r="D156" t="inlineStr">
         <is>
           <t>info@fischersneuart.de</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr">
         <is>
           <t>+49 6022 8512</t>
@@ -12221,14 +11961,11 @@
           <t>info@esh-meisterteam.de</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr"/>
       <c r="F157" t="inlineStr">
         <is>
           <t>06027 9905410</t>
         </is>
       </c>
-      <c r="G157" t="inlineStr"/>
-      <c r="H157" t="inlineStr"/>
       <c r="I157" t="inlineStr">
         <is>
           <t>Kleinostheim</t>
@@ -12281,7 +12018,6 @@
           <t>Elektriker</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr">
         <is>
           <t>hello@elfaisal.de</t>
@@ -12297,7 +12033,6 @@
           <t>+4915124259238</t>
         </is>
       </c>
-      <c r="G158" t="inlineStr"/>
       <c r="H158" t="inlineStr">
         <is>
           <t>63801</t>
@@ -12355,12 +12090,6 @@
           <t>Bauunternehmen</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr"/>
-      <c r="D159" t="inlineStr"/>
-      <c r="E159" t="inlineStr"/>
-      <c r="F159" t="inlineStr"/>
-      <c r="G159" t="inlineStr"/>
-      <c r="H159" t="inlineStr"/>
       <c r="I159" t="inlineStr">
         <is>
           <t>Kleinostheim</t>
@@ -12423,7 +12152,6 @@
           <t>info@schreinerei-wissel.de</t>
         </is>
       </c>
-      <c r="E160" t="inlineStr"/>
       <c r="F160" t="inlineStr">
         <is>
           <t>+49 6188 4486720</t>
@@ -12491,13 +12219,11 @@
           <t>Zimmerei / Schreinerei</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr">
         <is>
           <t>info@schreinerei-grebner.de</t>
         </is>
       </c>
-      <c r="E161" t="inlineStr"/>
       <c r="F161" t="inlineStr">
         <is>
           <t>+49 6188 5292</t>
@@ -12565,7 +12291,6 @@
           <t>Elektriker</t>
         </is>
       </c>
-      <c r="C162" t="inlineStr"/>
       <c r="D162" t="inlineStr">
         <is>
           <t>info@adlerelektro.de</t>
@@ -12643,20 +12368,16 @@
           <t>Sanitär / Heizung</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr"/>
       <c r="D163" t="inlineStr">
         <is>
           <t>info@heizungsanitaer-fuehrer.de</t>
         </is>
       </c>
-      <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr">
         <is>
           <t>06182 24785</t>
         </is>
       </c>
-      <c r="G163" t="inlineStr"/>
-      <c r="H163" t="inlineStr"/>
       <c r="I163" t="inlineStr">
         <is>
           <t>Karlstein am Main</t>
@@ -12719,14 +12440,11 @@
           <t>info@koloseus.de</t>
         </is>
       </c>
-      <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr">
         <is>
           <t>+49 6188 99530</t>
         </is>
       </c>
-      <c r="G164" t="inlineStr"/>
-      <c r="H164" t="inlineStr"/>
       <c r="I164" t="inlineStr">
         <is>
           <t>Karlstein am Main</t>
@@ -12861,13 +12579,11 @@
           <t>Dachdecker</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr"/>
       <c r="D166" t="inlineStr">
         <is>
           <t>info@dachdecker-herd.de</t>
         </is>
       </c>
-      <c r="E166" t="inlineStr"/>
       <c r="F166" t="inlineStr">
         <is>
           <t>+49 6023 1333</t>
@@ -12945,7 +12661,6 @@
           <t>info@emmel.de</t>
         </is>
       </c>
-      <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr">
         <is>
           <t>06023 9655-0</t>
@@ -13023,14 +12738,11 @@
           <t>schreinerei.amberg@t-online.de</t>
         </is>
       </c>
-      <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr">
         <is>
           <t>+49 6023 5488</t>
         </is>
       </c>
-      <c r="G168" t="inlineStr"/>
-      <c r="H168" t="inlineStr"/>
       <c r="I168" t="inlineStr">
         <is>
           <t>Alzenau</t>
@@ -13083,7 +12795,6 @@
           <t>Sanitär / Heizung</t>
         </is>
       </c>
-      <c r="C169" t="inlineStr"/>
       <c r="D169" t="inlineStr">
         <is>
           <t>info@bruder-haustechnik.de</t>
@@ -13099,8 +12810,6 @@
           <t>06182/22436</t>
         </is>
       </c>
-      <c r="G169" t="inlineStr"/>
-      <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr">
         <is>
           <t>Seligenstadt</t>
@@ -13173,8 +12882,6 @@
           <t>06182 826970</t>
         </is>
       </c>
-      <c r="G170" t="inlineStr"/>
-      <c r="H170" t="inlineStr"/>
       <c r="I170" t="inlineStr">
         <is>
           <t>Seligenstadt</t>
@@ -13232,15 +12939,11 @@
           <t>Matthias Hock</t>
         </is>
       </c>
-      <c r="D171" t="inlineStr"/>
-      <c r="E171" t="inlineStr"/>
       <c r="F171" t="inlineStr">
         <is>
           <t>06182-200121</t>
         </is>
       </c>
-      <c r="G171" t="inlineStr"/>
-      <c r="H171" t="inlineStr"/>
       <c r="I171" t="inlineStr">
         <is>
           <t>Seligenstadt</t>
@@ -13303,13 +13006,11 @@
           <t>info@schlosserei-millitzer-gmbh.de</t>
         </is>
       </c>
-      <c r="E172" t="inlineStr"/>
       <c r="F172" t="inlineStr">
         <is>
           <t>+49 6182 28123</t>
         </is>
       </c>
-      <c r="G172" t="inlineStr"/>
       <c r="H172" t="inlineStr">
         <is>
           <t>63500</t>
@@ -13377,14 +13078,11 @@
           <t>info@buehring-gmbh.com</t>
         </is>
       </c>
-      <c r="E173" t="inlineStr"/>
       <c r="F173" t="inlineStr">
         <is>
           <t>0 61 82 / 54 62</t>
         </is>
       </c>
-      <c r="G173" t="inlineStr"/>
-      <c r="H173" t="inlineStr"/>
       <c r="I173" t="inlineStr">
         <is>
           <t>Seligenstadt</t>
@@ -13437,7 +13135,6 @@
           <t>Sanitär / Heizung</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr">
         <is>
           <t>zentrale@rohrstar.de</t>
@@ -13453,8 +13150,6 @@
           <t>+49 6182 787787</t>
         </is>
       </c>
-      <c r="G174" t="inlineStr"/>
-      <c r="H174" t="inlineStr"/>
       <c r="I174" t="inlineStr">
         <is>
           <t>Seligenstadt</t>
@@ -13517,14 +13212,11 @@
           <t>info@purcraft.de</t>
         </is>
       </c>
-      <c r="E175" t="inlineStr"/>
       <c r="F175" t="inlineStr">
         <is>
           <t>+49 6182 772653-0</t>
         </is>
       </c>
-      <c r="G175" t="inlineStr"/>
-      <c r="H175" t="inlineStr"/>
       <c r="I175" t="inlineStr">
         <is>
           <t>Seligenstadt</t>
@@ -13597,8 +13289,6 @@
           <t>+49-6182-829047</t>
         </is>
       </c>
-      <c r="G176" t="inlineStr"/>
-      <c r="H176" t="inlineStr"/>
       <c r="I176" t="inlineStr">
         <is>
           <t>Seligenstadt</t>
@@ -13656,15 +13346,11 @@
           <t>Michael Winter</t>
         </is>
       </c>
-      <c r="D177" t="inlineStr"/>
-      <c r="E177" t="inlineStr"/>
       <c r="F177" t="inlineStr">
         <is>
           <t>+49(0)6182/7701600</t>
         </is>
       </c>
-      <c r="G177" t="inlineStr"/>
-      <c r="H177" t="inlineStr"/>
       <c r="I177" t="inlineStr">
         <is>
           <t>Seligenstadt</t>
@@ -13737,8 +13423,6 @@
           <t>06186 1734</t>
         </is>
       </c>
-      <c r="G178" t="inlineStr"/>
-      <c r="H178" t="inlineStr"/>
       <c r="I178" t="inlineStr">
         <is>
           <t>Hainburg</t>
@@ -13801,14 +13485,11 @@
           <t>info@kaelte-pietz.de</t>
         </is>
       </c>
-      <c r="E179" t="inlineStr"/>
       <c r="F179" t="inlineStr">
         <is>
           <t>06023 96800 200</t>
         </is>
       </c>
-      <c r="G179" t="inlineStr"/>
-      <c r="H179" t="inlineStr"/>
       <c r="I179" t="inlineStr">
         <is>
           <t>Hainburg</t>
@@ -13881,8 +13562,6 @@
           <t>+49 6181 300330</t>
         </is>
       </c>
-      <c r="G180" t="inlineStr"/>
-      <c r="H180" t="inlineStr"/>
       <c r="I180" t="inlineStr">
         <is>
           <t>Hanau</t>
@@ -13945,7 +13624,6 @@
           <t>info@kuerschner-kg.de</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr">
         <is>
           <t>+49 6181 79709</t>
@@ -14013,13 +13691,11 @@
           <t>Elektriker</t>
         </is>
       </c>
-      <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr">
         <is>
           <t>info@ets-schmidt.de</t>
         </is>
       </c>
-      <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr">
         <is>
           <t>+49 6181 3077866</t>
@@ -14097,7 +13773,6 @@
           <t>info@oetjen-gmbh.de</t>
         </is>
       </c>
-      <c r="E183" t="inlineStr"/>
       <c r="F183" t="inlineStr">
         <is>
           <t>+49 6181 575430</t>
@@ -14165,7 +13840,6 @@
           <t>Maler / Lackierer</t>
         </is>
       </c>
-      <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr">
         <is>
           <t>info@emmel-malerdesign.de</t>
@@ -14181,8 +13855,6 @@
           <t>+49 6181 71293</t>
         </is>
       </c>
-      <c r="G184" t="inlineStr"/>
-      <c r="H184" t="inlineStr"/>
       <c r="I184" t="inlineStr">
         <is>
           <t>Hanau</t>
@@ -14245,7 +13917,6 @@
           <t>info@amp-altbausanierung.de</t>
         </is>
       </c>
-      <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr">
         <is>
           <t>+49 6181 9060640</t>
@@ -14313,7 +13984,6 @@
           <t>Schreinerei</t>
         </is>
       </c>
-      <c r="C186" t="inlineStr"/>
       <c r="D186" t="inlineStr">
         <is>
           <t>info@schreinerei-ertelt.de</t>
@@ -14401,14 +14071,11 @@
           <t>info@viel-online.de</t>
         </is>
       </c>
-      <c r="E187" t="inlineStr"/>
       <c r="F187" t="inlineStr">
         <is>
           <t>+49 6183 3935</t>
         </is>
       </c>
-      <c r="G187" t="inlineStr"/>
-      <c r="H187" t="inlineStr"/>
       <c r="I187" t="inlineStr">
         <is>
           <t>Hanau</t>
@@ -14481,8 +14148,6 @@
           <t>+49 6181 364677 0</t>
         </is>
       </c>
-      <c r="G188" t="inlineStr"/>
-      <c r="H188" t="inlineStr"/>
       <c r="I188" t="inlineStr">
         <is>
           <t>Hanau</t>
@@ -14545,14 +14210,11 @@
           <t>info@struve-hanau.de</t>
         </is>
       </c>
-      <c r="E189" t="inlineStr"/>
       <c r="F189" t="inlineStr">
         <is>
           <t>+49618182077</t>
         </is>
       </c>
-      <c r="G189" t="inlineStr"/>
-      <c r="H189" t="inlineStr"/>
       <c r="I189" t="inlineStr">
         <is>
           <t>Hanau</t>
@@ -14697,7 +14359,6 @@
           <t>info@kraft-elektrobau.de</t>
         </is>
       </c>
-      <c r="E191" t="inlineStr"/>
       <c r="F191" t="inlineStr">
         <is>
           <t>+49 6181 97200</t>
@@ -14765,7 +14426,6 @@
           <t>Sanitär / Heizung</t>
         </is>
       </c>
-      <c r="C192" t="inlineStr"/>
       <c r="D192" t="inlineStr">
         <is>
           <t>info@abfluss-schaefer-gmbh.de</t>
@@ -14781,8 +14441,6 @@
           <t>+49 6183 9284200</t>
         </is>
       </c>
-      <c r="G192" t="inlineStr"/>
-      <c r="H192" t="inlineStr"/>
       <c r="I192" t="inlineStr">
         <is>
           <t>Hanau</t>
@@ -14917,7 +14575,6 @@
           <t>Heizung / Klima</t>
         </is>
       </c>
-      <c r="C194" t="inlineStr"/>
       <c r="D194" t="inlineStr">
         <is>
           <t>info@heck-gmbh.de</t>
@@ -14995,7 +14652,6 @@
           <t>Dachdecker</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr">
         <is>
           <t>info@schultheis-dach.de</t>
@@ -15011,8 +14667,6 @@
           <t>06181 / 9939-0</t>
         </is>
       </c>
-      <c r="G195" t="inlineStr"/>
-      <c r="H195" t="inlineStr"/>
       <c r="I195" t="inlineStr">
         <is>
           <t>Hanau</t>
@@ -15065,13 +14719,11 @@
           <t>Steinmetz</t>
         </is>
       </c>
-      <c r="C196" t="inlineStr"/>
       <c r="D196" t="inlineStr">
         <is>
           <t>mail@steinmetz-moeller.de</t>
         </is>
       </c>
-      <c r="E196" t="inlineStr"/>
       <c r="F196" t="inlineStr">
         <is>
           <t>06181/71355</t>
@@ -15139,7 +14791,6 @@
           <t>Heizung / Klima</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr">
         <is>
           <t>info@kaut.de</t>
@@ -15155,8 +14806,6 @@
           <t>+49 6109 69680</t>
         </is>
       </c>
-      <c r="G197" t="inlineStr"/>
-      <c r="H197" t="inlineStr"/>
       <c r="I197" t="inlineStr">
         <is>
           <t>Maintal</t>
@@ -15209,7 +14858,6 @@
           <t>Heizung / Klima</t>
         </is>
       </c>
-      <c r="C198" t="inlineStr"/>
       <c r="D198" t="inlineStr">
         <is>
           <t>data.privacy@copeland.com</t>
@@ -15225,8 +14873,6 @@
           <t>+49 6109 60590</t>
         </is>
       </c>
-      <c r="G198" t="inlineStr"/>
-      <c r="H198" t="inlineStr"/>
       <c r="I198" t="inlineStr">
         <is>
           <t>Maintal</t>
@@ -15299,8 +14945,6 @@
           <t>069 865661</t>
         </is>
       </c>
-      <c r="G199" t="inlineStr"/>
-      <c r="H199" t="inlineStr"/>
       <c r="I199" t="inlineStr">
         <is>
           <t>Maintal</t>
@@ -15353,20 +14997,16 @@
           <t>Steinmetz</t>
         </is>
       </c>
-      <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr">
         <is>
           <t>info@schneider-grabmale.com</t>
         </is>
       </c>
-      <c r="E200" t="inlineStr"/>
       <c r="F200" t="inlineStr">
         <is>
           <t>069 86 2002</t>
         </is>
       </c>
-      <c r="G200" t="inlineStr"/>
-      <c r="H200" t="inlineStr"/>
       <c r="I200" t="inlineStr">
         <is>
           <t>Maintal</t>
@@ -15419,13 +15059,11 @@
           <t>Zimmerei / Schreinerei</t>
         </is>
       </c>
-      <c r="C201" t="inlineStr"/>
       <c r="D201" t="inlineStr">
         <is>
           <t>info@boehm-schreinerei-glaserei.de</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr"/>
       <c r="F201" t="inlineStr">
         <is>
           <t>+49 6108 7969960</t>
@@ -15482,8 +15120,1341 @@
         </is>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Chmiel Bad- und Raum Design</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Fliesenleger</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Marek Chmiel-Kordylewski</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>fliesen.chmiel@gmail.com</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>+49 6108 791672</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Offenbacher Straße 8-10</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>63165</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Mühlheim am Main</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>https://www.chmiel-bad-raumdesign.de/</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>https://www.chmiel-bad-raumdesign.de/recht/impressum</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>Maintal</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>50.124361</t>
+        </is>
+      </c>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>8.831515</t>
+        </is>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>node/13704054823</t>
+        </is>
+      </c>
+      <c r="P202" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Eisen Ernst</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Schlüsseldienst</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>info@eisen-ernst.de</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>+49 69 671392</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Goldsteinstraße 3</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>60528</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>https://www.eisen-ernst.de/</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>https://www.eisen-ernst.de/kontakt/</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>50.085184</t>
+        </is>
+      </c>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>8.646981</t>
+        </is>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>node/632564596</t>
+        </is>
+      </c>
+      <c r="P203" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Hartmann Holzmarkt</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Schreinerei</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Astrid Fittje</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>info@hartmann-holzmarkt.de</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>+49 69 284001</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>https://hartmann-holzmarkt.de/</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>https://hartmann-holzmarkt.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>50.117409</t>
+        </is>
+      </c>
+      <c r="N204" t="inlineStr">
+        <is>
+          <t>8.685651</t>
+        </is>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>node/767279383</t>
+        </is>
+      </c>
+      <c r="P204" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Möller Feuerungstechnik GmbH</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Wolfgang Möller</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>info@moeller-feuerungstechnik.de</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>info@wesebo.de</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>069 / 56 20 88</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>https://www.moeller-feuerungstechnik.de/</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>https://moeller-feuerungstechnik.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>50.150025</t>
+        </is>
+      </c>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>8.680263</t>
+        </is>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>node/1796130484</t>
+        </is>
+      </c>
+      <c r="P205" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Friedrich Stier GmbH</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Friedrich Stier</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>info@stier-rolladen.de</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>+4969 55 59 12</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Ginnheimer Hohl 26</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>60431</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>https://www.stier-rolladen.de/</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>https://www.stier-rolladen.de/impressum.html</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>50.144433</t>
+        </is>
+      </c>
+      <c r="N206" t="inlineStr">
+        <is>
+          <t>8.651305</t>
+        </is>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>node/3116750705</t>
+        </is>
+      </c>
+      <c r="P206" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Steinmetz Kaufmann</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Steinmetz</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>David Prauschke</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>ak-stone@t-online.de</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>+49 6102 34875</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Friedhofstraße 53</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>63263</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>Neu-Isenburg</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>https://www.steinmetz-kaufmann.de/</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>https://steinmetz-kaufmann.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>50.048138</t>
+        </is>
+      </c>
+      <c r="N207" t="inlineStr">
+        <is>
+          <t>8.701947</t>
+        </is>
+      </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>node/3859405659</t>
+        </is>
+      </c>
+      <c r="P207" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Biergans</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Schlüsseldienst</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Marco Maier</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>info@biergans-sicherheit.de</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>https://www.biergans-sicherheit.de/</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>https://biergans-sicherheit.de/</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>50.047176</t>
+        </is>
+      </c>
+      <c r="N208" t="inlineStr">
+        <is>
+          <t>8.695573</t>
+        </is>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>node/4056576969</t>
+        </is>
+      </c>
+      <c r="P208" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Parkett &amp; Design</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Parkettleger</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>info@parkettunddesign.de</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>info@krifft.com</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>+49 176 96685840</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>https://www.parkettunddesign.de/</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>https://www.parkettunddesign.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>50.135541</t>
+        </is>
+      </c>
+      <c r="N209" t="inlineStr">
+        <is>
+          <t>8.764988</t>
+        </is>
+      </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>node/4075348054</t>
+        </is>
+      </c>
+      <c r="P209" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Schreinere Muth</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Zimmerei / Schreinerei</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Kai Muth</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>info@schreinerei-muth.de</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>+49 69 782747</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>https://www.schreinerei-muth.de/</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>https://schreinerei-muth.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>50.123009</t>
+        </is>
+      </c>
+      <c r="N210" t="inlineStr">
+        <is>
+          <t>8.596287</t>
+        </is>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>node/4087631683</t>
+        </is>
+      </c>
+      <c r="P210" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Müllers GmbH</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Heizung / Klima</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Gerald Maisch</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>kontakt@muellers-ffm.de</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>+49 69 787097</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>https://muellers-ffm.de/</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>https://muellers-ffm.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>50.124101</t>
+        </is>
+      </c>
+      <c r="N211" t="inlineStr">
+        <is>
+          <t>8.583002</t>
+        </is>
+      </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>node/4087677643</t>
+        </is>
+      </c>
+      <c r="P211" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Hartmann Fensterbau</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Fensterbau</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Willi Hartmann</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>info@fbhartmann.de</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>+49607374160</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>https://www.fb-h.de/</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>https://www.fb-h.de/</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>50.093024</t>
+        </is>
+      </c>
+      <c r="N212" t="inlineStr">
+        <is>
+          <t>8.751997</t>
+        </is>
+      </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>node/4094927509</t>
+        </is>
+      </c>
+      <c r="P212" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Mainfeuer</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Sanitär / Heizung</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>info@mainfeuer.de</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>06109 / 3 55 27</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>Triebstraße 2a - b</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>60388</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>https://www.mainfeuer.de/</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>https://www.mainfeuer.de/home/kontakt/</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>50.148735</t>
+        </is>
+      </c>
+      <c r="N213" t="inlineStr">
+        <is>
+          <t>8.753612</t>
+        </is>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>node/4204732970</t>
+        </is>
+      </c>
+      <c r="P213" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Grabdenkmale Knorr</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Steinmetz</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>beratung@knorr-grabdenkmale.de</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>info@wesebo.de</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>069/ 57 38 82</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>https://knorr-grabdenkmale.de/</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>https://knorr-grabdenkmale.de/kontakt/</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>50.160207</t>
+        </is>
+      </c>
+      <c r="N214" t="inlineStr">
+        <is>
+          <t>8.649702</t>
+        </is>
+      </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>node/5547534687</t>
+        </is>
+      </c>
+      <c r="P214" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Schusterlädchen &amp; Schlüsseldienst</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Schlüsseldienst</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Wolfgang Lenz</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>kontakt@schusterlaedchen.de</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>schusterlaedchen-w-lenz@t-online.de</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>+49 69 542875</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>https://www.schusterlaedchen.de/</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>https://www.schusterlaedchen.de/impressum</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>50.144394</t>
+        </is>
+      </c>
+      <c r="N215" t="inlineStr">
+        <is>
+          <t>8.693603</t>
+        </is>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>node/6385703483</t>
+        </is>
+      </c>
+      <c r="P215" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Frankfurter Schlüsseldienst</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Schlüsseldienst</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Cornelia Beek</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>kontakt@frankfurter-schluesseldienst.de</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>+49 69 28 20 05</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>Liebfrauenberg 39</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>60313</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>https://www.frankfurter-schluesseldienst.de/</t>
+        </is>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>https://www.frankfurter-schluesseldienst.de/impressum/</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>50.112501</t>
+        </is>
+      </c>
+      <c r="N216" t="inlineStr">
+        <is>
+          <t>8.681577</t>
+        </is>
+      </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>node/6424028949</t>
+        </is>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Anton Sonnenschutzsysteme GmbH</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Fensterbau</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Z. Naftaliev</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>info@anton-gmbh.de</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>+49 69 780 780</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>https://anton-gmbh.de/</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>https://www.anton-gmbh.de/impressum</t>
+        </is>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>50.122560</t>
+        </is>
+      </c>
+      <c r="N217" t="inlineStr">
+        <is>
+          <t>8.635478</t>
+        </is>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>node/7983965649</t>
+        </is>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Schlosserei von Kessler</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Metallbau</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>mvk64@gmx.de</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>+49 69 672678</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>http://www.schlosserei-von-kessler.de</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>http://www.schlosserei-von-kessler.de/</t>
+        </is>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>50.088194</t>
+        </is>
+      </c>
+      <c r="N218" t="inlineStr">
+        <is>
+          <t>8.642147</t>
+        </is>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>node/7985888982</t>
+        </is>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>nur E-Mail</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Teppichreinigung Runte</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Zimmerei / Schreinerei</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Thomas Runte</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>anfrage@runte-teppichreinigung.de</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>06181-94990</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>https://www.runte-teppichreinigung.de</t>
+        </is>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>https://www.runte-teppichreinigung.de/impressum</t>
+        </is>
+      </c>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>50.149527</t>
+        </is>
+      </c>
+      <c r="N219" t="inlineStr">
+        <is>
+          <t>8.620136</t>
+        </is>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>node/8253648961</t>
+        </is>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Schreinerei Lott</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Schreinerei</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Manfred Lott</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>lott.schreinerei@t-online.de</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>+49 69 518051</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Alt-Eschersheim 40</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>60433</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>https://www.schreinerei-lott.de/</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>https://www.schreinerei-lott.de/</t>
+        </is>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>50.160479</t>
+        </is>
+      </c>
+      <c r="N220" t="inlineStr">
+        <is>
+          <t>8.655680</t>
+        </is>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>node/8266502605</t>
+        </is>
+      </c>
+      <c r="P220" t="inlineStr">
+        <is>
+          <t>vollständig</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P201"/>
+  <autoFilter ref="A1:P220"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>